<commit_message>
Queda independiente los rotation history y solo el admin puede ver el rotation history de los dos entornos
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -8006,6 +8006,81 @@
       <c r="CY11" s="10" t="n">
         <v>5</v>
       </c>
+      <c r="ASX11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASY11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASZ11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATA11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATB11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATC11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATD11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATE11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATF11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATG11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATH11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATI11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATJ11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATK11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATL11" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" thickBot="1">
       <c r="A12" t="inlineStr">
@@ -9216,6 +9291,41 @@
         </is>
       </c>
       <c r="ARY15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASW15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASX15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASY15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ASZ15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATA15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATB15" s="21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ATC15" s="21" t="inlineStr">
         <is>
           <t>ON</t>
         </is>

</xml_diff>

<commit_message>
se soluciona conflicto de horas
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1423,4 +1423,297 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100CA9322843C908448A7CC4C80959E7EA5" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="61007b38270afa745228085cb2122e93">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ac1a3513-d81a-4c18-8050-a999882817d8" xmlns:ns3="8005b84f-6d40-4948-b2ef-cdf217df6c3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5de3a4fc5895f375d6ccd08492f33264" ns2:_="" ns3:_="">
+    <xsd:import namespace="ac1a3513-d81a-4c18-8050-a999882817d8"/>
+    <xsd:import namespace="8005b84f-6d40-4948-b2ef-cdf217df6c3a"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ac1a3513-d81a-4c18-8050-a999882817d8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="13" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="16" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="181d9607-3483-4463-b74c-937ca49446f0" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8005b84f-6d40-4948-b2ef-cdf217df6c3a" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{81d9232d-8d15-47ec-b722-159594258bdf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="8005b84f-6d40-4948-b2ef-cdf217df6c3a">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="22" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="23" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8005b84f-6d40-4948-b2ef-cdf217df6c3a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac1a3513-d81a-4c18-8050-a999882817d8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1342A764-2469-4015-B9BA-F35AEE725421}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2413D28A-FDF4-4BB2-8960-30323CE67359}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53D49827-0FD6-42E4-84D2-1F1D5E79F373}"/>
 </file>
</xml_diff>

<commit_message>
se hace correccion de las eliminaciones y se hace eliminacion en cascada BD, Excel
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EE18"/>
+  <dimension ref="A1:EP18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,6 +919,39 @@
       <c r="EE1" s="1" t="n">
         <v>45935</v>
       </c>
+      <c r="EF1" s="1" t="n">
+        <v>45979</v>
+      </c>
+      <c r="EG1" s="1" t="n">
+        <v>45980</v>
+      </c>
+      <c r="EH1" s="1" t="n">
+        <v>45981</v>
+      </c>
+      <c r="EI1" s="1" t="n">
+        <v>45982</v>
+      </c>
+      <c r="EJ1" s="1" t="n">
+        <v>45983</v>
+      </c>
+      <c r="EK1" s="1" t="n">
+        <v>45984</v>
+      </c>
+      <c r="EL1" s="1" t="n">
+        <v>45985</v>
+      </c>
+      <c r="EM1" s="1" t="n">
+        <v>45986</v>
+      </c>
+      <c r="EN1" s="1" t="n">
+        <v>45987</v>
+      </c>
+      <c r="EO1" s="1" t="n">
+        <v>45988</v>
+      </c>
+      <c r="EP1" s="1" t="n">
+        <v>45989</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -936,6 +969,61 @@
           <t>NM00007</t>
         </is>
       </c>
+      <c r="EF2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EG2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EH2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EI2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EJ2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EK2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EO2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EP2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -1324,6 +1412,61 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>TESTEDIT</t>
+        </is>
+      </c>
+      <c r="EF17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EG17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EH17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EI17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EJ17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EK17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EL17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EM17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EN17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EO17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EP17" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1423,297 +1566,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100CA9322843C908448A7CC4C80959E7EA5" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="61007b38270afa745228085cb2122e93">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ac1a3513-d81a-4c18-8050-a999882817d8" xmlns:ns3="8005b84f-6d40-4948-b2ef-cdf217df6c3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5de3a4fc5895f375d6ccd08492f33264" ns2:_="" ns3:_="">
-    <xsd:import namespace="ac1a3513-d81a-4c18-8050-a999882817d8"/>
-    <xsd:import namespace="8005b84f-6d40-4948-b2ef-cdf217df6c3a"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ac1a3513-d81a-4c18-8050-a999882817d8" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="13" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="16" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="181d9607-3483-4463-b74c-937ca49446f0" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8005b84f-6d40-4948-b2ef-cdf217df6c3a" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{81d9232d-8d15-47ec-b722-159594258bdf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="8005b84f-6d40-4948-b2ef-cdf217df6c3a">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="22" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="23" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8005b84f-6d40-4948-b2ef-cdf217df6c3a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac1a3513-d81a-4c18-8050-a999882817d8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1342A764-2469-4015-B9BA-F35AEE725421}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2413D28A-FDF4-4BB2-8960-30323CE67359}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53D49827-0FD6-42E4-84D2-1F1D5E79F373}"/>
 </file>
</xml_diff>

<commit_message>
asignacion por dropdown esta funcional pero se debe de corregir la hora que esta tomando de los shift porque esta diferente al de la ventana de opcion 1  y tambien se debe colocar funcional el scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EP18"/>
+  <dimension ref="A1:EW18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -952,6 +952,27 @@
       <c r="EP1" s="1" t="n">
         <v>45989</v>
       </c>
+      <c r="EQ1" s="1" t="n">
+        <v>45996</v>
+      </c>
+      <c r="ER1" s="1" t="n">
+        <v>45997</v>
+      </c>
+      <c r="ES1" s="1" t="n">
+        <v>45998</v>
+      </c>
+      <c r="ET1" s="1" t="n">
+        <v>45999</v>
+      </c>
+      <c r="EU1" s="1" t="n">
+        <v>46000</v>
+      </c>
+      <c r="EV1" s="1" t="n">
+        <v>46001</v>
+      </c>
+      <c r="EW1" s="1" t="n">
+        <v>46002</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -1024,13 +1045,44 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="EQ2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ER2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ES2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ET2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EU2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EV2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EW2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fuel attendant</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Aloekoe Figaro</t>
@@ -1039,6 +1091,11 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>NM00009</t>
+        </is>
+      </c>
+      <c r="ER3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Soluciona inconsistencia visual donde los días se ordenaban como texto en lugar de fecha, provocando saltos de mes erróneos en la vista previa.
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,72 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\PLG\inboundoutboundGit\inboundoutbound\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDFB9BA-5FF0-4A4C-8452-D8E6EC06B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>TEAM</t>
-  </si>
-  <si>
-    <t>ROLE</t>
-  </si>
-  <si>
-    <t>NAME</t>
-  </si>
-  <si>
-    <t>BADGE</t>
-  </si>
-  <si>
-    <t>Miguel Venegas</t>
-  </si>
-  <si>
-    <t>NM00001</t>
-  </si>
-  <si>
-    <t>ON</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -75,6 +39,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,24 +60,85 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -395,498 +426,591 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FC2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:FI3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:159" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>BADGE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n">
         <v>44735</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1" s="1" t="n">
         <v>44736</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1" s="1" t="n">
         <v>44737</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1" s="1" t="n">
         <v>44738</v>
       </c>
-      <c r="I1" s="1">
+      <c r="I1" s="1" t="n">
         <v>44739</v>
       </c>
-      <c r="J1" s="1">
+      <c r="J1" s="1" t="n">
         <v>44740</v>
       </c>
-      <c r="K1" s="1">
+      <c r="K1" s="1" t="n">
         <v>44741</v>
       </c>
-      <c r="L1" s="1">
+      <c r="L1" s="1" t="n">
         <v>44742</v>
       </c>
-      <c r="M1" s="1">
+      <c r="M1" s="1" t="n">
         <v>44743</v>
       </c>
-      <c r="N1" s="1">
+      <c r="N1" s="1" t="n">
         <v>44744</v>
       </c>
-      <c r="O1" s="1">
+      <c r="O1" s="1" t="n">
         <v>44745</v>
       </c>
-      <c r="P1" s="1">
+      <c r="P1" s="1" t="n">
         <v>44746</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="Q1" s="1" t="n">
         <v>44747</v>
       </c>
-      <c r="R1" s="1">
+      <c r="R1" s="1" t="n">
         <v>44748</v>
       </c>
-      <c r="S1" s="1">
+      <c r="S1" s="1" t="n">
         <v>44749</v>
       </c>
-      <c r="T1" s="1">
+      <c r="T1" s="1" t="n">
         <v>44750</v>
       </c>
-      <c r="U1" s="1">
+      <c r="U1" s="1" t="n">
         <v>44751</v>
       </c>
-      <c r="V1" s="1">
+      <c r="V1" s="1" t="n">
         <v>44752</v>
       </c>
-      <c r="W1" s="1">
+      <c r="W1" s="1" t="n">
         <v>44753</v>
       </c>
-      <c r="X1" s="1">
+      <c r="X1" s="1" t="n">
         <v>44754</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="Y1" s="1" t="n">
         <v>44755</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Z1" s="1" t="n">
         <v>44756</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AA1" s="1" t="n">
         <v>44757</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AB1" s="1" t="n">
         <v>44758</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AC1" s="1" t="n">
         <v>44759</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AD1" s="1" t="n">
         <v>44760</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AE1" s="1" t="n">
         <v>44761</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AF1" s="1" t="n">
         <v>44762</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AG1" s="1" t="n">
         <v>44763</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AH1" s="1" t="n">
         <v>44764</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="AI1" s="1" t="n">
         <v>44765</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AJ1" s="1" t="n">
         <v>44766</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AK1" s="1" t="n">
         <v>44767</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AL1" s="1" t="n">
         <v>44768</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AM1" s="1" t="n">
         <v>44769</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AN1" s="1" t="n">
         <v>44770</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AO1" s="1" t="n">
         <v>44771</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AP1" s="1" t="n">
         <v>44772</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AQ1" s="1" t="n">
         <v>44773</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AR1" s="1" t="n">
         <v>44774</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AS1" s="1" t="n">
         <v>44775</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AT1" s="1" t="n">
         <v>44776</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AU1" s="1" t="n">
         <v>44777</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AV1" s="1" t="n">
         <v>44778</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AW1" s="1" t="n">
         <v>44779</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AX1" s="1" t="n">
         <v>44780</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AY1" s="1" t="n">
         <v>44781</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AZ1" s="1" t="n">
         <v>44782</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="BA1" s="1" t="n">
         <v>44783</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="BB1" s="1" t="n">
         <v>44784</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="BC1" s="1" t="n">
         <v>44785</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="BD1" s="1" t="n">
         <v>44786</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="BE1" s="1" t="n">
         <v>44787</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="BF1" s="1" t="n">
         <v>44788</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="BG1" s="1" t="n">
         <v>44789</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="BH1" s="1" t="n">
         <v>44790</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="BI1" s="1" t="n">
         <v>44791</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BJ1" s="1" t="n">
         <v>44792</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BK1" s="1" t="n">
         <v>44793</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BL1" s="1" t="n">
         <v>44794</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BM1" s="1" t="n">
         <v>44795</v>
       </c>
-      <c r="BN1" s="1">
+      <c r="BN1" s="1" t="n">
         <v>44796</v>
       </c>
-      <c r="BO1" s="1">
+      <c r="BO1" s="1" t="n">
         <v>44797</v>
       </c>
-      <c r="BP1" s="1">
+      <c r="BP1" s="1" t="n">
         <v>44798</v>
       </c>
-      <c r="BQ1" s="1">
+      <c r="BQ1" s="1" t="n">
         <v>44799</v>
       </c>
-      <c r="BR1" s="1">
+      <c r="BR1" s="1" t="n">
         <v>44800</v>
       </c>
-      <c r="BS1" s="1">
+      <c r="BS1" s="1" t="n">
         <v>44801</v>
       </c>
-      <c r="BT1" s="1">
+      <c r="BT1" s="1" t="n">
         <v>44802</v>
       </c>
-      <c r="BU1" s="1">
+      <c r="BU1" s="1" t="n">
         <v>44803</v>
       </c>
-      <c r="BV1" s="1">
+      <c r="BV1" s="1" t="n">
         <v>44804</v>
       </c>
-      <c r="BW1" s="1">
+      <c r="BW1" s="1" t="n">
         <v>44805</v>
       </c>
-      <c r="BX1" s="1">
+      <c r="BX1" s="1" t="n">
         <v>44806</v>
       </c>
-      <c r="BY1" s="1">
+      <c r="BY1" s="1" t="n">
         <v>44807</v>
       </c>
-      <c r="BZ1" s="1">
+      <c r="BZ1" s="1" t="n">
         <v>44808</v>
       </c>
-      <c r="CA1" s="1">
+      <c r="CA1" s="1" t="n">
         <v>44809</v>
       </c>
-      <c r="CB1" s="1">
+      <c r="CB1" s="1" t="n">
         <v>44810</v>
       </c>
-      <c r="CC1" s="1">
+      <c r="CC1" s="1" t="n">
         <v>44811</v>
       </c>
-      <c r="CD1" s="1">
+      <c r="CD1" s="1" t="n">
         <v>44812</v>
       </c>
-      <c r="CE1" s="1">
+      <c r="CE1" s="1" t="n">
         <v>44813</v>
       </c>
-      <c r="CF1" s="1">
+      <c r="CF1" s="1" t="n">
         <v>44814</v>
       </c>
-      <c r="CG1" s="1">
+      <c r="CG1" s="1" t="n">
         <v>44815</v>
       </c>
-      <c r="CH1" s="1">
+      <c r="CH1" s="1" t="n">
         <v>44816</v>
       </c>
-      <c r="CI1" s="1">
+      <c r="CI1" s="1" t="n">
         <v>44817</v>
       </c>
-      <c r="CJ1" s="1">
+      <c r="CJ1" s="1" t="n">
         <v>44818</v>
       </c>
-      <c r="CK1" s="1">
+      <c r="CK1" s="1" t="n">
         <v>44819</v>
       </c>
-      <c r="CL1" s="1">
+      <c r="CL1" s="1" t="n">
         <v>44820</v>
       </c>
-      <c r="CM1" s="1">
+      <c r="CM1" s="1" t="n">
         <v>44821</v>
       </c>
-      <c r="CN1" s="1">
+      <c r="CN1" s="1" t="n">
         <v>44822</v>
       </c>
-      <c r="CO1" s="1">
+      <c r="CO1" s="1" t="n">
         <v>44823</v>
       </c>
-      <c r="CP1" s="1">
+      <c r="CP1" s="1" t="n">
         <v>44824</v>
       </c>
-      <c r="CQ1" s="1">
+      <c r="CQ1" s="1" t="n">
         <v>44825</v>
       </c>
-      <c r="CR1" s="1">
+      <c r="CR1" s="1" t="n">
         <v>44826</v>
       </c>
-      <c r="CS1" s="1">
+      <c r="CS1" s="1" t="n">
         <v>44827</v>
       </c>
-      <c r="CT1" s="1">
+      <c r="CT1" s="1" t="n">
         <v>44828</v>
       </c>
-      <c r="CU1" s="1">
+      <c r="CU1" s="1" t="n">
         <v>44829</v>
       </c>
-      <c r="CV1" s="1">
+      <c r="CV1" s="1" t="n">
         <v>44830</v>
       </c>
-      <c r="CW1" s="1">
+      <c r="CW1" s="1" t="n">
         <v>44831</v>
       </c>
-      <c r="CX1" s="1">
+      <c r="CX1" s="1" t="n">
         <v>44832</v>
       </c>
-      <c r="CY1" s="1">
+      <c r="CY1" s="1" t="n">
         <v>44833</v>
       </c>
-      <c r="CZ1" s="1">
+      <c r="CZ1" s="1" t="n">
         <v>44834</v>
       </c>
-      <c r="DA1" s="1">
+      <c r="DA1" s="1" t="n">
         <v>45898</v>
       </c>
-      <c r="DB1" s="1">
+      <c r="DB1" s="1" t="n">
         <v>45899</v>
       </c>
-      <c r="DC1" s="1">
+      <c r="DC1" s="1" t="n">
         <v>45900</v>
       </c>
-      <c r="DD1" s="1">
+      <c r="DD1" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="DE1" s="1">
+      <c r="DE1" s="1" t="n">
         <v>45902</v>
       </c>
-      <c r="DF1" s="1">
+      <c r="DF1" s="1" t="n">
         <v>45903</v>
       </c>
-      <c r="DG1" s="1">
+      <c r="DG1" s="1" t="n">
         <v>45909</v>
       </c>
-      <c r="DH1" s="1">
+      <c r="DH1" s="1" t="n">
         <v>45910</v>
       </c>
-      <c r="DI1" s="1">
+      <c r="DI1" s="1" t="n">
         <v>45911</v>
       </c>
-      <c r="DJ1" s="1">
+      <c r="DJ1" s="1" t="n">
         <v>45912</v>
       </c>
-      <c r="DK1" s="1">
+      <c r="DK1" s="1" t="n">
         <v>45913</v>
       </c>
-      <c r="DL1" s="1">
+      <c r="DL1" s="1" t="n">
         <v>45914</v>
       </c>
-      <c r="DM1" s="1">
+      <c r="DM1" s="1" t="n">
         <v>45915</v>
       </c>
-      <c r="DN1" s="1">
+      <c r="DN1" s="1" t="n">
         <v>45918</v>
       </c>
-      <c r="DO1" s="1">
+      <c r="DO1" s="1" t="n">
         <v>45919</v>
       </c>
-      <c r="DP1" s="1">
+      <c r="DP1" s="1" t="n">
         <v>45920</v>
       </c>
-      <c r="DQ1" s="1">
+      <c r="DQ1" s="1" t="n">
         <v>45921</v>
       </c>
-      <c r="DR1" s="1">
+      <c r="DR1" s="1" t="n">
         <v>45922</v>
       </c>
-      <c r="DS1" s="1">
+      <c r="DS1" s="1" t="n">
         <v>45923</v>
       </c>
-      <c r="DT1" s="1">
+      <c r="DT1" s="1" t="n">
         <v>45924</v>
       </c>
-      <c r="DU1" s="1">
+      <c r="DU1" s="1" t="n">
         <v>45926</v>
       </c>
-      <c r="DV1" s="1">
+      <c r="DV1" s="1" t="n">
         <v>45927</v>
       </c>
-      <c r="DW1" s="1">
+      <c r="DW1" s="1" t="n">
         <v>45928</v>
       </c>
-      <c r="DX1" s="1">
+      <c r="DX1" s="1" t="n">
         <v>45929</v>
       </c>
-      <c r="DY1" s="1">
+      <c r="DY1" s="1" t="n">
         <v>45925</v>
       </c>
-      <c r="DZ1" s="1">
+      <c r="DZ1" s="1" t="n">
         <v>45930</v>
       </c>
-      <c r="EA1" s="1">
+      <c r="EA1" s="1" t="n">
         <v>45931</v>
       </c>
-      <c r="EB1" s="1">
+      <c r="EB1" s="1" t="n">
         <v>45932</v>
       </c>
-      <c r="EC1" s="1">
+      <c r="EC1" s="1" t="n">
         <v>45933</v>
       </c>
-      <c r="ED1" s="1">
+      <c r="ED1" s="1" t="n">
         <v>45934</v>
       </c>
-      <c r="EE1" s="1">
+      <c r="EE1" s="1" t="n">
         <v>45935</v>
       </c>
-      <c r="EF1" s="1">
+      <c r="EF1" s="1" t="n">
         <v>45979</v>
       </c>
-      <c r="EG1" s="1">
+      <c r="EG1" s="1" t="n">
         <v>45980</v>
       </c>
-      <c r="EH1" s="1">
+      <c r="EH1" s="1" t="n">
         <v>45981</v>
       </c>
-      <c r="EI1" s="1">
+      <c r="EI1" s="1" t="n">
         <v>45982</v>
       </c>
-      <c r="EJ1" s="1">
+      <c r="EJ1" s="1" t="n">
         <v>45983</v>
       </c>
-      <c r="EK1" s="1">
+      <c r="EK1" s="1" t="n">
         <v>45984</v>
       </c>
-      <c r="EL1" s="1">
+      <c r="EL1" s="1" t="n">
         <v>45985</v>
       </c>
-      <c r="EM1" s="1">
+      <c r="EM1" s="1" t="n">
         <v>45986</v>
       </c>
-      <c r="EN1" s="1">
+      <c r="EN1" s="1" t="n">
         <v>45987</v>
       </c>
-      <c r="EO1" s="1">
+      <c r="EO1" s="1" t="n">
         <v>45988</v>
       </c>
-      <c r="EP1" s="1">
+      <c r="EP1" s="1" t="n">
         <v>45989</v>
       </c>
-      <c r="EQ1" s="1">
+      <c r="EQ1" s="1" t="n">
         <v>45996</v>
       </c>
-      <c r="ER1" s="1">
+      <c r="ER1" s="1" t="n">
         <v>45997</v>
       </c>
-      <c r="ES1" s="1">
+      <c r="ES1" s="1" t="n">
         <v>45998</v>
       </c>
-      <c r="ET1" s="1">
+      <c r="ET1" s="1" t="n">
         <v>45999</v>
       </c>
-      <c r="EU1" s="1">
+      <c r="EU1" s="1" t="n">
         <v>46000</v>
       </c>
-      <c r="EV1" s="1">
+      <c r="EV1" s="1" t="n">
         <v>46001</v>
       </c>
-      <c r="EW1" s="1">
+      <c r="EW1" s="1" t="n">
         <v>46002</v>
       </c>
-      <c r="EX1" s="1">
+      <c r="EX1" s="1" t="n">
         <v>45990</v>
       </c>
-      <c r="EY1" s="1">
+      <c r="EY1" s="1" t="n">
         <v>45991</v>
       </c>
-      <c r="EZ1" s="1">
+      <c r="EZ1" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="FA1" s="1">
+      <c r="FA1" s="1" t="n">
         <v>45993</v>
       </c>
-      <c r="FB1" s="1">
+      <c r="FB1" s="1" t="n">
         <v>45994</v>
       </c>
-      <c r="FC1" s="1">
+      <c r="FC1" s="1" t="n">
         <v>45995</v>
       </c>
+      <c r="FD1" s="3" t="n">
+        <v>46003</v>
+      </c>
+      <c r="FE1" s="3" t="n">
+        <v>46004</v>
+      </c>
+      <c r="FF1" s="3" t="n">
+        <v>46005</v>
+      </c>
+      <c r="FG1" s="3" t="n">
+        <v>46006</v>
+      </c>
+      <c r="FH1" s="3" t="n">
+        <v>46007</v>
+      </c>
+      <c r="FI1" s="3" t="n">
+        <v>46008</v>
+      </c>
     </row>
-    <row r="2" spans="1:159" x14ac:dyDescent="0.3">
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="EU2" s="2" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Miguel Venegas</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NM00001</t>
+        </is>
+      </c>
+      <c r="EU2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Kevin Blanco</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A123</t>
+        </is>
+      </c>
+      <c r="EV3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="EW3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FD3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FE3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FF3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FG3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FH3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FI3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se soluciona problema de hhora en el scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -28,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
         <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,12 +66,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -957,11 +964,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fuel Attendant</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Kevin Blanco</t>
@@ -972,6 +975,21 @@
           <t>A123</t>
         </is>
       </c>
+      <c r="EQ3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ER3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="ES3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="EV3" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
@@ -980,6 +998,26 @@
       <c r="EW3" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
+        </is>
+      </c>
+      <c r="EZ3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FA3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FB3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FC3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
       <c r="FD3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
se solucional el bug que cuando se hacia el scroll right no se visualizaba el role en la pantalla de Plan Staff
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FI3"/>
+  <dimension ref="A1:FR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -945,109 +945,382 @@
       <c r="FI1" s="3" t="n">
         <v>46008</v>
       </c>
+      <c r="FJ1" s="3" t="n">
+        <v>46029</v>
+      </c>
+      <c r="FK1" s="3" t="n">
+        <v>46030</v>
+      </c>
+      <c r="FL1" s="3" t="n">
+        <v>46031</v>
+      </c>
+      <c r="FM1" s="3" t="n">
+        <v>46032</v>
+      </c>
+      <c r="FN1" s="3" t="n">
+        <v>46033</v>
+      </c>
+      <c r="FO1" s="3" t="n">
+        <v>46034</v>
+      </c>
+      <c r="FP1" s="3" t="n">
+        <v>46035</v>
+      </c>
+      <c r="FQ1" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="FR1" s="3" t="n">
+        <v>46037</v>
+      </c>
     </row>
     <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Miguel Venegas</t>
+          <t>Anibal Rodriguez Fuentes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NM00001</t>
-        </is>
-      </c>
-      <c r="EU2" s="2" t="inlineStr">
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="EU2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EV2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EW2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FD2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FE2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FF2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FG2" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FH2" s="5" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kevin Blanco</t>
+          <t>Ricardo Gomez</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A123</t>
-        </is>
-      </c>
-      <c r="EQ3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="ER3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="ES3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="EV3" s="4" t="inlineStr">
+          <t>A147</t>
+        </is>
+      </c>
+      <c r="EV3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="EW3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FD3" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Yiseth Castro</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A357</t>
+        </is>
+      </c>
+      <c r="FJ4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FK4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FL4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FM4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FN4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FO4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FP4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FQ4" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Jorge Silva</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>S413</t>
+        </is>
+      </c>
+      <c r="FJ5" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="EW3" s="4" t="inlineStr">
+      <c r="FK5" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="EZ3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FA3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FB3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FC3" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FD3" s="4" t="inlineStr">
+      <c r="FL5" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="FE3" s="4" t="inlineStr">
+      <c r="FM5" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="FF3" s="4" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Andres Lopez</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A460</t>
+        </is>
+      </c>
+      <c r="FJ6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FK6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FL6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FM6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FN6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FO6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FP6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FQ6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FR6" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fernando Herrara</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>A463</t>
+        </is>
+      </c>
+      <c r="FJ7" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FK7" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FL7" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FM7" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FN7" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Camila Vargas</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>M791</t>
+        </is>
+      </c>
+      <c r="FJ8" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="FG3" s="4" t="inlineStr">
+      <c r="FK8" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="FH3" s="4" t="inlineStr">
+      <c r="FL8" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="FI3" s="4" t="inlineStr">
+      <c r="FM8" s="4" t="inlineStr">
         <is>
           <t>ON NS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Carlo Mendez</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>S412</t>
+        </is>
+      </c>
+      <c r="FN9" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FO9" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FP9" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FQ9" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se soluciona conflicto de asignacion de pick up drop off y Remark mostrando el dato en la ventana flotante e inboundoutbound
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -28,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFAA00"/>
+        <bgColor rgb="00FFAA00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,13 +72,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -147,6 +154,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="FL3" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-14:00</t>
+      </text>
+    </comment>
+    <comment ref="FM3" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-14:00</t>
+      </text>
+    </comment>
+    <comment ref="FN3" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-14:00</t>
+      </text>
+    </comment>
+    <comment ref="FO3" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-14:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -438,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FR9"/>
+  <dimension ref="A1:FR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1029,6 +1066,31 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="FK2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FL2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FM2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FN2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="FO2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -1061,6 +1123,26 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="FL3" s="6" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="FM3" s="6" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="FN3" s="6" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="FO3" s="6" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -1155,6 +1237,26 @@
           <t>ON NS</t>
         </is>
       </c>
+      <c r="FN5" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FO5" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FP5" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FQ5" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -1256,69 +1358,37 @@
       </c>
     </row>
     <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Camila Vargas</t>
+          <t>Carlo Mendez</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M791</t>
-        </is>
-      </c>
-      <c r="FJ8" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="FK8" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="FL8" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="FM8" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Supervisor</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Carlo Mendez</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
           <t>S412</t>
         </is>
       </c>
-      <c r="FN9" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FO9" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FP9" s="5" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="FQ9" s="5" t="inlineStr">
+      <c r="FN8" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FO8" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FP8" s="5" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="FQ8" s="5" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -1326,5 +1396,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correcion entry y exito por scroll right
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -760,6 +760,51 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -823,6 +868,31 @@
         </is>
       </c>
       <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>

</xml_diff>

<commit_message>
SCROLL Right estable en los dos enornos y OFF consistente Se realiza prueba de generacion de reporte y es acorde a la informacion del excel plan staff
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -15,9 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -28,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -39,6 +38,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,11 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ3"/>
+  <dimension ref="A1:CJ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -451,31 +464,31 @@
           <t>BADGE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" s="2" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" s="2" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" s="2" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" s="2" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" s="2" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="2" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" s="2" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="N1" s="2" t="n">
@@ -712,12 +725,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fernando Herrera</t>
+          <t>Andres Lopez</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A463</t>
+          <t>A460</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -750,16 +763,16 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
@@ -771,36 +784,6 @@
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Z2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -814,87 +797,131 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Fernando Herrera</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A463</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Aldair Hernandez</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>A147</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="X3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Z3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AA3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AB3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Site Manager</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Miguel Venegas</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PK789</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
correccion final del software
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,66 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\PLG\inboundoutboundGit\inboundoutbound\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA35858-7091-4CB9-B47F-D12EC060FB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>TEAM</t>
-  </si>
-  <si>
-    <t>ROLE</t>
-  </si>
-  <si>
-    <t>NAME</t>
-  </si>
-  <si>
-    <t>BADGE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF2AFF"/>
+        <bgColor rgb="00FF2AFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -75,24 +59,150 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -379,280 +489,427 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CJ1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CJ3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:88" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>BADGE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1" s="1" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1" s="1" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1" s="1" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="1">
+      <c r="I1" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="1">
+      <c r="J1" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="1">
+      <c r="K1" s="1" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="1">
+      <c r="L1" s="1" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="1">
+      <c r="M1" s="1" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="1">
+      <c r="N1" s="1" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="1">
+      <c r="O1" s="1" t="n">
         <v>46039</v>
       </c>
-      <c r="P1" s="1">
+      <c r="P1" s="1" t="n">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="Q1" s="1" t="n">
         <v>46041</v>
       </c>
-      <c r="R1" s="1">
+      <c r="R1" s="1" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="1">
+      <c r="S1" s="1" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="1">
+      <c r="T1" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="1">
+      <c r="U1" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="1">
+      <c r="V1" s="1" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="1">
+      <c r="W1" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="1">
+      <c r="X1" s="1" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="Y1" s="1" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Z1" s="1" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AA1" s="1" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AB1" s="1" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AC1" s="1" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AD1" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AE1" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AF1" s="1" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AG1" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AH1" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="AI1" s="1" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AJ1" s="1" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AK1" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AL1" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AM1" s="1" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AN1" s="1" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AO1" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AP1" s="1" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AQ1" s="1" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AR1" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AS1" s="1" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AT1" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AU1" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AV1" s="1" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AW1" s="1" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AX1" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AY1" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AZ1" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="BA1" s="1" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="BB1" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="BC1" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="BD1" s="1" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="BE1" s="1" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="BF1" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="BG1" s="1" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="BH1" s="1" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="BI1" s="1" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BJ1" s="1" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BK1" s="1" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BL1" s="1" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BM1" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1">
+      <c r="BN1" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1">
+      <c r="BO1" s="1" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1">
+      <c r="BP1" s="1" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1">
+      <c r="BQ1" s="1" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1">
+      <c r="BR1" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1">
+      <c r="BS1" s="1" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1">
+      <c r="BT1" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1">
+      <c r="BU1" s="1" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1">
+      <c r="BV1" s="1" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1">
+      <c r="BW1" s="1" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1">
+      <c r="BX1" s="1" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1">
+      <c r="BY1" s="1" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1">
+      <c r="BZ1" s="1" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1">
+      <c r="CA1" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1">
+      <c r="CB1" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1">
+      <c r="CC1" s="1" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1">
+      <c r="CD1" s="1" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1">
+      <c r="CE1" s="1" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1">
+      <c r="CF1" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1">
+      <c r="CG1" s="1" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1">
+      <c r="CH1" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1">
+      <c r="CI1" s="1" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1">
+      <c r="CJ1" s="1" t="n">
         <v>46112</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KP789</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Aldair Hernandez</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KP321</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se generan opciones paralelas a OFF creadas desde el menu de turnos
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,30 @@
         <bgColor rgb="00FF2AFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00550000"/>
+        <bgColor rgb="00550000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF5500"/>
+        <bgColor rgb="00FF5500"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,11 +83,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -166,39 +194,24 @@
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
+    <comment ref="O3" authorId="0" shapeId="0">
       <text>
-        <t>13:00-17:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0">
+    <comment ref="P3" authorId="0" shapeId="0">
       <text>
-        <t>13:00-17:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0">
+    <comment ref="Q3" authorId="0" shapeId="0">
       <text>
-        <t>13:00-17:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0">
+    <comment ref="R3" authorId="0" shapeId="0">
       <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="I3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="K3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
+        <t>00:00-00:00</t>
       </text>
     </comment>
   </commentList>
@@ -872,39 +885,44 @@
           <t>KP321</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>SUS</t>
+        </is>
+      </c>
+      <c r="U3" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="V3" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="W3" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="X3" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
caracteristica  paralela de off en la UI UX
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -194,6 +194,31 @@
         <t>13:00-17:00</t>
       </text>
     </comment>
+    <comment ref="Y2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AA2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AB2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AC2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
     <comment ref="O3" authorId="0" shapeId="0">
       <text>
         <t>00:00-00:00</t>
@@ -868,6 +893,31 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
Barra de carga por concepto de hilo
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -235,6 +235,21 @@
       </text>
     </comment>
     <comment ref="R3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AD3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AE3" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="AF3" authorId="0" shapeId="0">
       <text>
         <t>00:00-00:00</t>
       </text>
@@ -975,6 +990,21 @@
           <t>OFF</t>
         </is>
       </c>
+      <c r="AD3" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="AE3" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="AF3" s="4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Drag optimizado con refresh instantaneo
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,12 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -92,6 +98,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -174,84 +181,24 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
+    <comment ref="K3" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="F2" authorId="0" shapeId="0">
+    <comment ref="L3" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="G2" authorId="0" shapeId="0">
+    <comment ref="M3" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
       </text>
     </comment>
-    <comment ref="H2" authorId="0" shapeId="0">
+    <comment ref="N3" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="Y2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="Z2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AA2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AB2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AC2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="O3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="P3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="Q3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="R3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AD3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AE3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="AF3" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
       </text>
     </comment>
   </commentList>
@@ -843,42 +790,32 @@
           <t>KP789</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -888,6 +825,16 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
@@ -896,41 +843,6 @@
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Y2" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="Z2" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AA2" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AB2" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AC2" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
         </is>
       </c>
     </row>
@@ -950,59 +862,24 @@
           <t>KP321</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
-        <is>
-          <t>SUS</t>
-        </is>
-      </c>
-      <c r="P3" s="6" t="inlineStr">
-        <is>
-          <t>SUS</t>
-        </is>
-      </c>
-      <c r="Q3" s="6" t="inlineStr">
-        <is>
-          <t>SUS</t>
-        </is>
-      </c>
-      <c r="R3" s="6" t="inlineStr">
-        <is>
-          <t>SUS</t>
-        </is>
-      </c>
-      <c r="U3" s="7" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="V3" s="7" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="W3" s="7" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="X3" s="7" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="AD3" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AE3" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
-        </is>
-      </c>
-      <c r="AF3" s="4" t="inlineStr">
-        <is>
-          <t>LV</t>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Implementacion de UI moderna y correccion de Theme
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -882,6 +882,31 @@
           <t>INT</t>
         </is>
       </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
se soluciona problema de star date con drag utilizando left_col + 1
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -89,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +100,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -173,36 +175,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>ShiftType</author>
-  </authors>
-  <commentList>
-    <comment ref="K3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="L3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="M3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="N3" authorId="0" shapeId="0">
-      <text>
-        <t>13:00-17:00</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -494,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ3"/>
+  <dimension ref="A1:CP3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -773,6 +745,24 @@
       <c r="CJ1" s="1" t="n">
         <v>46112</v>
       </c>
+      <c r="CK1" s="9" t="n">
+        <v>46023</v>
+      </c>
+      <c r="CL1" s="9" t="n">
+        <v>46024</v>
+      </c>
+      <c r="CM1" s="9" t="n">
+        <v>46025</v>
+      </c>
+      <c r="CN1" s="9" t="n">
+        <v>46026</v>
+      </c>
+      <c r="CO1" s="9" t="n">
+        <v>46027</v>
+      </c>
+      <c r="CP1" s="9" t="n">
+        <v>46028</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -790,57 +780,32 @@
           <t>KP789</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="CK2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CL2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CM2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CN2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CO2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CP2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -862,29 +827,33 @@
           <t>KP321</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>INT</t>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se soluciona problema  de drag utilizando  el left_col + 1
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -181,6 +181,31 @@
     <author>ShiftType</author>
   </authors>
   <commentList>
+    <comment ref="V2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="Y2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0" shapeId="0">
+      <text>
+        <t>13:00-17:00</t>
+      </text>
+    </comment>
     <comment ref="K3" authorId="0" shapeId="0">
       <text>
         <t>13:00-17:00</t>
@@ -845,6 +870,31 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
different color in the weekend and Mon, Tues, Wed in header
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP3"/>
+  <dimension ref="A1:EY3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -763,6 +763,189 @@
       <c r="CP1" s="9" t="n">
         <v>46028</v>
       </c>
+      <c r="CQ1" s="9" t="n">
+        <v>46113</v>
+      </c>
+      <c r="CR1" s="9" t="n">
+        <v>46114</v>
+      </c>
+      <c r="CS1" s="9" t="n">
+        <v>46115</v>
+      </c>
+      <c r="CT1" s="9" t="n">
+        <v>46116</v>
+      </c>
+      <c r="CU1" s="9" t="n">
+        <v>46117</v>
+      </c>
+      <c r="CV1" s="9" t="n">
+        <v>46118</v>
+      </c>
+      <c r="CW1" s="9" t="n">
+        <v>46119</v>
+      </c>
+      <c r="CX1" s="9" t="n">
+        <v>46120</v>
+      </c>
+      <c r="CY1" s="9" t="n">
+        <v>46121</v>
+      </c>
+      <c r="CZ1" s="9" t="n">
+        <v>46122</v>
+      </c>
+      <c r="DA1" s="9" t="n">
+        <v>46123</v>
+      </c>
+      <c r="DB1" s="9" t="n">
+        <v>46124</v>
+      </c>
+      <c r="DC1" s="9" t="n">
+        <v>46125</v>
+      </c>
+      <c r="DD1" s="9" t="n">
+        <v>46126</v>
+      </c>
+      <c r="DE1" s="9" t="n">
+        <v>46127</v>
+      </c>
+      <c r="DF1" s="9" t="n">
+        <v>46128</v>
+      </c>
+      <c r="DG1" s="9" t="n">
+        <v>46129</v>
+      </c>
+      <c r="DH1" s="9" t="n">
+        <v>46130</v>
+      </c>
+      <c r="DI1" s="9" t="n">
+        <v>46131</v>
+      </c>
+      <c r="DJ1" s="9" t="n">
+        <v>46132</v>
+      </c>
+      <c r="DK1" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="DL1" s="9" t="n">
+        <v>46134</v>
+      </c>
+      <c r="DM1" s="9" t="n">
+        <v>46135</v>
+      </c>
+      <c r="DN1" s="9" t="n">
+        <v>46136</v>
+      </c>
+      <c r="DO1" s="9" t="n">
+        <v>46137</v>
+      </c>
+      <c r="DP1" s="9" t="n">
+        <v>46138</v>
+      </c>
+      <c r="DQ1" s="9" t="n">
+        <v>46139</v>
+      </c>
+      <c r="DR1" s="9" t="n">
+        <v>46140</v>
+      </c>
+      <c r="DS1" s="9" t="n">
+        <v>46141</v>
+      </c>
+      <c r="DT1" s="9" t="n">
+        <v>46142</v>
+      </c>
+      <c r="DU1" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="DV1" s="9" t="n">
+        <v>46144</v>
+      </c>
+      <c r="DW1" s="9" t="n">
+        <v>46145</v>
+      </c>
+      <c r="DX1" s="9" t="n">
+        <v>46146</v>
+      </c>
+      <c r="DY1" s="9" t="n">
+        <v>46147</v>
+      </c>
+      <c r="DZ1" s="9" t="n">
+        <v>46148</v>
+      </c>
+      <c r="EA1" s="9" t="n">
+        <v>46149</v>
+      </c>
+      <c r="EB1" s="9" t="n">
+        <v>46150</v>
+      </c>
+      <c r="EC1" s="9" t="n">
+        <v>46151</v>
+      </c>
+      <c r="ED1" s="9" t="n">
+        <v>46152</v>
+      </c>
+      <c r="EE1" s="9" t="n">
+        <v>46153</v>
+      </c>
+      <c r="EF1" s="9" t="n">
+        <v>46154</v>
+      </c>
+      <c r="EG1" s="9" t="n">
+        <v>46155</v>
+      </c>
+      <c r="EH1" s="9" t="n">
+        <v>46156</v>
+      </c>
+      <c r="EI1" s="9" t="n">
+        <v>46157</v>
+      </c>
+      <c r="EJ1" s="9" t="n">
+        <v>46158</v>
+      </c>
+      <c r="EK1" s="9" t="n">
+        <v>46159</v>
+      </c>
+      <c r="EL1" s="9" t="n">
+        <v>46160</v>
+      </c>
+      <c r="EM1" s="9" t="n">
+        <v>46161</v>
+      </c>
+      <c r="EN1" s="9" t="n">
+        <v>46162</v>
+      </c>
+      <c r="EO1" s="9" t="n">
+        <v>46163</v>
+      </c>
+      <c r="EP1" s="9" t="n">
+        <v>46164</v>
+      </c>
+      <c r="EQ1" s="9" t="n">
+        <v>46165</v>
+      </c>
+      <c r="ER1" s="9" t="n">
+        <v>46166</v>
+      </c>
+      <c r="ES1" s="9" t="n">
+        <v>46167</v>
+      </c>
+      <c r="ET1" s="9" t="n">
+        <v>46168</v>
+      </c>
+      <c r="EU1" s="9" t="n">
+        <v>46169</v>
+      </c>
+      <c r="EV1" s="9" t="n">
+        <v>46170</v>
+      </c>
+      <c r="EW1" s="9" t="n">
+        <v>46171</v>
+      </c>
+      <c r="EX1" s="9" t="n">
+        <v>46172</v>
+      </c>
+      <c r="EY1" s="9" t="n">
+        <v>46173</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
el usuario tiene una ventana exclusiva para el role
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,81 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\inboundoutbound\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B366859-1AA9-4C7D-AEB8-E2382EE59D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>TEAM</t>
+  </si>
+  <si>
+    <t>ROLE</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>BADGE</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF2AFF"/>
-        <bgColor rgb="00FF2AFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00550000"/>
-        <bgColor rgb="00550000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF5500"/>
-        <bgColor rgb="00FF5500"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -90,90 +75,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -461,594 +380,478 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:EY3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:EY1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
+    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ROLE</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>NAME</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>BADGE</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="n">
+    <row r="1" spans="1:155" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1">
         <v>46029</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" s="1">
         <v>46030</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" s="1">
         <v>46031</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" s="1">
         <v>46032</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" s="1">
         <v>46033</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" s="1">
         <v>46034</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="1">
         <v>46035</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" s="1">
         <v>46036</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" s="1">
         <v>46037</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" s="1">
         <v>46038</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" s="1">
         <v>46039</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" s="1">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" s="1">
         <v>46041</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" s="1">
         <v>46042</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" s="1">
         <v>46043</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" s="1">
         <v>46044</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" s="1">
         <v>46045</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" s="1">
         <v>46046</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" s="1">
         <v>46047</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" s="1">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" s="1">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" s="1">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" s="1">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" s="1">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" s="1">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" s="1">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" s="1">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" s="1">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" s="1">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" s="1">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" s="1">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" s="1">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" s="1">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" s="1">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" s="1">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" s="1">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" s="1">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" s="1">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" s="1">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" s="1">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" s="1">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" s="1">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" s="1">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" s="1">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1" t="n">
+      <c r="AW1" s="1">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1" t="n">
+      <c r="AX1" s="1">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1" t="n">
+      <c r="AY1" s="1">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1" t="n">
+      <c r="AZ1" s="1">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1" t="n">
+      <c r="BA1" s="1">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1" t="n">
+      <c r="BB1" s="1">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1" t="n">
+      <c r="BC1" s="1">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1" t="n">
+      <c r="BD1" s="1">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1" t="n">
+      <c r="BE1" s="1">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1" t="n">
+      <c r="BF1" s="1">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1" t="n">
+      <c r="BG1" s="1">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1" t="n">
+      <c r="BH1" s="1">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1" t="n">
+      <c r="BI1" s="1">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1" t="n">
+      <c r="BJ1" s="1">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1" t="n">
+      <c r="BK1" s="1">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1" t="n">
+      <c r="BL1" s="1">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1" t="n">
+      <c r="BM1" s="1">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1" t="n">
+      <c r="BN1" s="1">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1" t="n">
+      <c r="BO1" s="1">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1" t="n">
+      <c r="BP1" s="1">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1" t="n">
+      <c r="BQ1" s="1">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1" t="n">
+      <c r="BR1" s="1">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1" t="n">
+      <c r="BS1" s="1">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1" t="n">
+      <c r="BT1" s="1">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1" t="n">
+      <c r="BU1" s="1">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1" t="n">
+      <c r="BV1" s="1">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1" t="n">
+      <c r="BW1" s="1">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1" t="n">
+      <c r="BX1" s="1">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1" t="n">
+      <c r="BY1" s="1">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1" t="n">
+      <c r="BZ1" s="1">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1" t="n">
+      <c r="CA1" s="1">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1" t="n">
+      <c r="CB1" s="1">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1" t="n">
+      <c r="CC1" s="1">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1" t="n">
+      <c r="CD1" s="1">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1" t="n">
+      <c r="CE1" s="1">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1" t="n">
+      <c r="CF1" s="1">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1" t="n">
+      <c r="CG1" s="1">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1" t="n">
+      <c r="CH1" s="1">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1" t="n">
+      <c r="CI1" s="1">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1" t="n">
+      <c r="CJ1" s="1">
         <v>46112</v>
       </c>
-      <c r="CK1" s="9" t="n">
+      <c r="CK1" s="2">
         <v>46023</v>
       </c>
-      <c r="CL1" s="9" t="n">
+      <c r="CL1" s="2">
         <v>46024</v>
       </c>
-      <c r="CM1" s="9" t="n">
+      <c r="CM1" s="2">
         <v>46025</v>
       </c>
-      <c r="CN1" s="9" t="n">
+      <c r="CN1" s="2">
         <v>46026</v>
       </c>
-      <c r="CO1" s="9" t="n">
+      <c r="CO1" s="2">
         <v>46027</v>
       </c>
-      <c r="CP1" s="9" t="n">
+      <c r="CP1" s="2">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="9" t="n">
+      <c r="CQ1" s="2">
         <v>46113</v>
       </c>
-      <c r="CR1" s="9" t="n">
+      <c r="CR1" s="2">
         <v>46114</v>
       </c>
-      <c r="CS1" s="9" t="n">
+      <c r="CS1" s="2">
         <v>46115</v>
       </c>
-      <c r="CT1" s="9" t="n">
+      <c r="CT1" s="2">
         <v>46116</v>
       </c>
-      <c r="CU1" s="9" t="n">
+      <c r="CU1" s="2">
         <v>46117</v>
       </c>
-      <c r="CV1" s="9" t="n">
+      <c r="CV1" s="2">
         <v>46118</v>
       </c>
-      <c r="CW1" s="9" t="n">
+      <c r="CW1" s="2">
         <v>46119</v>
       </c>
-      <c r="CX1" s="9" t="n">
+      <c r="CX1" s="2">
         <v>46120</v>
       </c>
-      <c r="CY1" s="9" t="n">
+      <c r="CY1" s="2">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="9" t="n">
+      <c r="CZ1" s="2">
         <v>46122</v>
       </c>
-      <c r="DA1" s="9" t="n">
+      <c r="DA1" s="2">
         <v>46123</v>
       </c>
-      <c r="DB1" s="9" t="n">
+      <c r="DB1" s="2">
         <v>46124</v>
       </c>
-      <c r="DC1" s="9" t="n">
+      <c r="DC1" s="2">
         <v>46125</v>
       </c>
-      <c r="DD1" s="9" t="n">
+      <c r="DD1" s="2">
         <v>46126</v>
       </c>
-      <c r="DE1" s="9" t="n">
+      <c r="DE1" s="2">
         <v>46127</v>
       </c>
-      <c r="DF1" s="9" t="n">
+      <c r="DF1" s="2">
         <v>46128</v>
       </c>
-      <c r="DG1" s="9" t="n">
+      <c r="DG1" s="2">
         <v>46129</v>
       </c>
-      <c r="DH1" s="9" t="n">
+      <c r="DH1" s="2">
         <v>46130</v>
       </c>
-      <c r="DI1" s="9" t="n">
+      <c r="DI1" s="2">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="9" t="n">
+      <c r="DJ1" s="2">
         <v>46132</v>
       </c>
-      <c r="DK1" s="9" t="n">
+      <c r="DK1" s="2">
         <v>46133</v>
       </c>
-      <c r="DL1" s="9" t="n">
+      <c r="DL1" s="2">
         <v>46134</v>
       </c>
-      <c r="DM1" s="9" t="n">
+      <c r="DM1" s="2">
         <v>46135</v>
       </c>
-      <c r="DN1" s="9" t="n">
+      <c r="DN1" s="2">
         <v>46136</v>
       </c>
-      <c r="DO1" s="9" t="n">
+      <c r="DO1" s="2">
         <v>46137</v>
       </c>
-      <c r="DP1" s="9" t="n">
+      <c r="DP1" s="2">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="9" t="n">
+      <c r="DQ1" s="2">
         <v>46139</v>
       </c>
-      <c r="DR1" s="9" t="n">
+      <c r="DR1" s="2">
         <v>46140</v>
       </c>
-      <c r="DS1" s="9" t="n">
+      <c r="DS1" s="2">
         <v>46141</v>
       </c>
-      <c r="DT1" s="9" t="n">
+      <c r="DT1" s="2">
         <v>46142</v>
       </c>
-      <c r="DU1" s="9" t="n">
+      <c r="DU1" s="2">
         <v>46143</v>
       </c>
-      <c r="DV1" s="9" t="n">
+      <c r="DV1" s="2">
         <v>46144</v>
       </c>
-      <c r="DW1" s="9" t="n">
+      <c r="DW1" s="2">
         <v>46145</v>
       </c>
-      <c r="DX1" s="9" t="n">
+      <c r="DX1" s="2">
         <v>46146</v>
       </c>
-      <c r="DY1" s="9" t="n">
+      <c r="DY1" s="2">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="9" t="n">
+      <c r="DZ1" s="2">
         <v>46148</v>
       </c>
-      <c r="EA1" s="9" t="n">
+      <c r="EA1" s="2">
         <v>46149</v>
       </c>
-      <c r="EB1" s="9" t="n">
+      <c r="EB1" s="2">
         <v>46150</v>
       </c>
-      <c r="EC1" s="9" t="n">
+      <c r="EC1" s="2">
         <v>46151</v>
       </c>
-      <c r="ED1" s="9" t="n">
+      <c r="ED1" s="2">
         <v>46152</v>
       </c>
-      <c r="EE1" s="9" t="n">
+      <c r="EE1" s="2">
         <v>46153</v>
       </c>
-      <c r="EF1" s="9" t="n">
+      <c r="EF1" s="2">
         <v>46154</v>
       </c>
-      <c r="EG1" s="9" t="n">
+      <c r="EG1" s="2">
         <v>46155</v>
       </c>
-      <c r="EH1" s="9" t="n">
+      <c r="EH1" s="2">
         <v>46156</v>
       </c>
-      <c r="EI1" s="9" t="n">
+      <c r="EI1" s="2">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="9" t="n">
+      <c r="EJ1" s="2">
         <v>46158</v>
       </c>
-      <c r="EK1" s="9" t="n">
+      <c r="EK1" s="2">
         <v>46159</v>
       </c>
-      <c r="EL1" s="9" t="n">
+      <c r="EL1" s="2">
         <v>46160</v>
       </c>
-      <c r="EM1" s="9" t="n">
+      <c r="EM1" s="2">
         <v>46161</v>
       </c>
-      <c r="EN1" s="9" t="n">
+      <c r="EN1" s="2">
         <v>46162</v>
       </c>
-      <c r="EO1" s="9" t="n">
+      <c r="EO1" s="2">
         <v>46163</v>
       </c>
-      <c r="EP1" s="9" t="n">
+      <c r="EP1" s="2">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="9" t="n">
+      <c r="EQ1" s="2">
         <v>46165</v>
       </c>
-      <c r="ER1" s="9" t="n">
+      <c r="ER1" s="2">
         <v>46166</v>
       </c>
-      <c r="ES1" s="9" t="n">
+      <c r="ES1" s="2">
         <v>46167</v>
       </c>
-      <c r="ET1" s="9" t="n">
+      <c r="ET1" s="2">
         <v>46168</v>
       </c>
-      <c r="EU1" s="9" t="n">
+      <c r="EU1" s="2">
         <v>46169</v>
       </c>
-      <c r="EV1" s="9" t="n">
+      <c r="EV1" s="2">
         <v>46170</v>
       </c>
-      <c r="EW1" s="9" t="n">
+      <c r="EW1" s="2">
         <v>46171</v>
       </c>
-      <c r="EX1" s="9" t="n">
+      <c r="EX1" s="2">
         <v>46172</v>
       </c>
-      <c r="EY1" s="9" t="n">
+      <c r="EY1" s="2">
         <v>46173</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Fuel Attendant</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Juan Perez</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>KP789</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CO2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CP2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Supervisor</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Aldair Hernandez</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>KP321</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Guardando cambios en improvingDrag
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,66 +1,56 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\inboundoutbound\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B366859-1AA9-4C7D-AEB8-E2382EE59D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>TEAM</t>
-  </si>
-  <si>
-    <t>ROLE</t>
-  </si>
-  <si>
-    <t>NAME</t>
-  </si>
-  <si>
-    <t>BADGE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0055007F"/>
+        <bgColor rgb="0055007F"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -75,25 +65,112 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-09:00</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-09:00</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-09:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -380,481 +457,566 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EY1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:EY2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:155" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>BADGE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1" s="2" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1" s="2" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1" s="2" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="1">
+      <c r="I1" s="2" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="1">
+      <c r="J1" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="1">
+      <c r="K1" s="2" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="1">
+      <c r="L1" s="2" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="1">
+      <c r="M1" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="1">
+      <c r="N1" s="2" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="1">
+      <c r="O1" s="2" t="n">
         <v>46039</v>
       </c>
-      <c r="P1" s="1">
+      <c r="P1" s="2" t="n">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="Q1" s="2" t="n">
         <v>46041</v>
       </c>
-      <c r="R1" s="1">
+      <c r="R1" s="2" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="1">
+      <c r="S1" s="2" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="1">
+      <c r="T1" s="2" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="1">
+      <c r="U1" s="2" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="1">
+      <c r="V1" s="2" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="1">
+      <c r="W1" s="2" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="1">
+      <c r="X1" s="2" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="Y1" s="2" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Z1" s="2" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AA1" s="2" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AB1" s="2" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AC1" s="2" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AD1" s="2" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AE1" s="2" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AF1" s="2" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AG1" s="2" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AH1" s="2" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="AI1" s="2" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AJ1" s="2" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AK1" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AL1" s="2" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AM1" s="2" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AN1" s="2" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AO1" s="2" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AP1" s="2" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AQ1" s="2" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AR1" s="2" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AS1" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AT1" s="2" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AU1" s="2" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AV1" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AW1" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AX1" s="2" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AY1" s="2" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AZ1" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="BA1" s="2" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="BB1" s="2" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="BC1" s="2" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="BD1" s="2" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="BE1" s="2" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="BF1" s="2" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="BG1" s="2" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="BH1" s="2" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="BI1" s="2" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BJ1" s="2" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BK1" s="2" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BL1" s="2" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BM1" s="2" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1">
+      <c r="BN1" s="2" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1">
+      <c r="BO1" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1">
+      <c r="BP1" s="2" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1">
+      <c r="BQ1" s="2" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1">
+      <c r="BR1" s="2" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1">
+      <c r="BS1" s="2" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1">
+      <c r="BT1" s="2" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1">
+      <c r="BU1" s="2" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1">
+      <c r="BV1" s="2" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1">
+      <c r="BW1" s="2" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1">
+      <c r="BX1" s="2" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1">
+      <c r="BY1" s="2" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1">
+      <c r="BZ1" s="2" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1">
+      <c r="CA1" s="2" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1">
+      <c r="CB1" s="2" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1">
+      <c r="CC1" s="2" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1">
+      <c r="CD1" s="2" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1">
+      <c r="CE1" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1">
+      <c r="CF1" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1">
+      <c r="CG1" s="2" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1">
+      <c r="CH1" s="2" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1">
+      <c r="CI1" s="2" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1">
+      <c r="CJ1" s="2" t="n">
         <v>46112</v>
       </c>
-      <c r="CK1" s="2">
+      <c r="CK1" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="CL1" s="2">
+      <c r="CL1" s="2" t="n">
         <v>46024</v>
       </c>
-      <c r="CM1" s="2">
+      <c r="CM1" s="2" t="n">
         <v>46025</v>
       </c>
-      <c r="CN1" s="2">
+      <c r="CN1" s="2" t="n">
         <v>46026</v>
       </c>
-      <c r="CO1" s="2">
+      <c r="CO1" s="2" t="n">
         <v>46027</v>
       </c>
-      <c r="CP1" s="2">
+      <c r="CP1" s="2" t="n">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="2">
+      <c r="CQ1" s="2" t="n">
         <v>46113</v>
       </c>
-      <c r="CR1" s="2">
+      <c r="CR1" s="2" t="n">
         <v>46114</v>
       </c>
-      <c r="CS1" s="2">
+      <c r="CS1" s="2" t="n">
         <v>46115</v>
       </c>
-      <c r="CT1" s="2">
+      <c r="CT1" s="2" t="n">
         <v>46116</v>
       </c>
-      <c r="CU1" s="2">
+      <c r="CU1" s="2" t="n">
         <v>46117</v>
       </c>
-      <c r="CV1" s="2">
+      <c r="CV1" s="2" t="n">
         <v>46118</v>
       </c>
-      <c r="CW1" s="2">
+      <c r="CW1" s="2" t="n">
         <v>46119</v>
       </c>
-      <c r="CX1" s="2">
+      <c r="CX1" s="2" t="n">
         <v>46120</v>
       </c>
-      <c r="CY1" s="2">
+      <c r="CY1" s="2" t="n">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="2">
+      <c r="CZ1" s="2" t="n">
         <v>46122</v>
       </c>
-      <c r="DA1" s="2">
+      <c r="DA1" s="2" t="n">
         <v>46123</v>
       </c>
-      <c r="DB1" s="2">
+      <c r="DB1" s="2" t="n">
         <v>46124</v>
       </c>
-      <c r="DC1" s="2">
+      <c r="DC1" s="2" t="n">
         <v>46125</v>
       </c>
-      <c r="DD1" s="2">
+      <c r="DD1" s="2" t="n">
         <v>46126</v>
       </c>
-      <c r="DE1" s="2">
+      <c r="DE1" s="2" t="n">
         <v>46127</v>
       </c>
-      <c r="DF1" s="2">
+      <c r="DF1" s="2" t="n">
         <v>46128</v>
       </c>
-      <c r="DG1" s="2">
+      <c r="DG1" s="2" t="n">
         <v>46129</v>
       </c>
-      <c r="DH1" s="2">
+      <c r="DH1" s="2" t="n">
         <v>46130</v>
       </c>
-      <c r="DI1" s="2">
+      <c r="DI1" s="2" t="n">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="2">
+      <c r="DJ1" s="2" t="n">
         <v>46132</v>
       </c>
-      <c r="DK1" s="2">
+      <c r="DK1" s="2" t="n">
         <v>46133</v>
       </c>
-      <c r="DL1" s="2">
+      <c r="DL1" s="2" t="n">
         <v>46134</v>
       </c>
-      <c r="DM1" s="2">
+      <c r="DM1" s="2" t="n">
         <v>46135</v>
       </c>
-      <c r="DN1" s="2">
+      <c r="DN1" s="2" t="n">
         <v>46136</v>
       </c>
-      <c r="DO1" s="2">
+      <c r="DO1" s="2" t="n">
         <v>46137</v>
       </c>
-      <c r="DP1" s="2">
+      <c r="DP1" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="2">
+      <c r="DQ1" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="DR1" s="2">
+      <c r="DR1" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="DS1" s="2">
+      <c r="DS1" s="2" t="n">
         <v>46141</v>
       </c>
-      <c r="DT1" s="2">
+      <c r="DT1" s="2" t="n">
         <v>46142</v>
       </c>
-      <c r="DU1" s="2">
+      <c r="DU1" s="2" t="n">
         <v>46143</v>
       </c>
-      <c r="DV1" s="2">
+      <c r="DV1" s="2" t="n">
         <v>46144</v>
       </c>
-      <c r="DW1" s="2">
+      <c r="DW1" s="2" t="n">
         <v>46145</v>
       </c>
-      <c r="DX1" s="2">
+      <c r="DX1" s="2" t="n">
         <v>46146</v>
       </c>
-      <c r="DY1" s="2">
+      <c r="DY1" s="2" t="n">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="2">
+      <c r="DZ1" s="2" t="n">
         <v>46148</v>
       </c>
-      <c r="EA1" s="2">
+      <c r="EA1" s="2" t="n">
         <v>46149</v>
       </c>
-      <c r="EB1" s="2">
+      <c r="EB1" s="2" t="n">
         <v>46150</v>
       </c>
-      <c r="EC1" s="2">
+      <c r="EC1" s="2" t="n">
         <v>46151</v>
       </c>
-      <c r="ED1" s="2">
+      <c r="ED1" s="2" t="n">
         <v>46152</v>
       </c>
-      <c r="EE1" s="2">
+      <c r="EE1" s="2" t="n">
         <v>46153</v>
       </c>
-      <c r="EF1" s="2">
+      <c r="EF1" s="2" t="n">
         <v>46154</v>
       </c>
-      <c r="EG1" s="2">
+      <c r="EG1" s="2" t="n">
         <v>46155</v>
       </c>
-      <c r="EH1" s="2">
+      <c r="EH1" s="2" t="n">
         <v>46156</v>
       </c>
-      <c r="EI1" s="2">
+      <c r="EI1" s="2" t="n">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="2">
+      <c r="EJ1" s="2" t="n">
         <v>46158</v>
       </c>
-      <c r="EK1" s="2">
+      <c r="EK1" s="2" t="n">
         <v>46159</v>
       </c>
-      <c r="EL1" s="2">
+      <c r="EL1" s="2" t="n">
         <v>46160</v>
       </c>
-      <c r="EM1" s="2">
+      <c r="EM1" s="2" t="n">
         <v>46161</v>
       </c>
-      <c r="EN1" s="2">
+      <c r="EN1" s="2" t="n">
         <v>46162</v>
       </c>
-      <c r="EO1" s="2">
+      <c r="EO1" s="2" t="n">
         <v>46163</v>
       </c>
-      <c r="EP1" s="2">
+      <c r="EP1" s="2" t="n">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="2">
+      <c r="EQ1" s="2" t="n">
         <v>46165</v>
       </c>
-      <c r="ER1" s="2">
+      <c r="ER1" s="2" t="n">
         <v>46166</v>
       </c>
-      <c r="ES1" s="2">
+      <c r="ES1" s="2" t="n">
         <v>46167</v>
       </c>
-      <c r="ET1" s="2">
+      <c r="ET1" s="2" t="n">
         <v>46168</v>
       </c>
-      <c r="EU1" s="2">
+      <c r="EU1" s="2" t="n">
         <v>46169</v>
       </c>
-      <c r="EV1" s="2">
+      <c r="EV1" s="2" t="n">
         <v>46170</v>
       </c>
-      <c r="EW1" s="2">
+      <c r="EW1" s="2" t="n">
         <v>46171</v>
       </c>
-      <c r="EX1" s="2">
+      <c r="EX1" s="2" t="n">
         <v>46172</v>
       </c>
-      <c r="EY1" s="2">
+      <c r="EY1" s="2" t="n">
         <v>46173</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Miguel Venecas</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>L169</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CK2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CL2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CM2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CN2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CO2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CP2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Smart Drag Totalmente Funcional
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -165,6 +165,11 @@
       </text>
     </comment>
     <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>06:00-09:00</t>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="0" shapeId="0">
       <text>
         <t>06:00-09:00</t>
       </text>
@@ -974,12 +979,67 @@
           <t>HD</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Al cambiar de Role ya se actualiza el view del schedule
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY2"/>
+  <dimension ref="A1:EY3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -934,6 +934,38 @@
           <t>E786</t>
         </is>
       </c>
+      <c r="AL2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fuel Attendant</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Elver Gonzales</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KL569</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Inicio de solucion a popup colision
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -36,20 +36,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0055007F"/>
-        <bgColor rgb="0055007F"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,13 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY3"/>
+  <dimension ref="A1:EY2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -464,506 +456,534 @@
           <t>BADGE</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n">
+      <c r="E1" s="1" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="F1" s="1" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="1" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="H1" s="1" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="I1" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="2" t="n">
+      <c r="K1" s="1" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="2" t="n">
+      <c r="L1" s="1" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="2" t="n">
+      <c r="M1" s="1" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="2" t="n">
+      <c r="N1" s="1" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="2" t="n">
+      <c r="O1" s="1" t="n">
         <v>46039</v>
       </c>
-      <c r="P1" s="2" t="n">
+      <c r="P1" s="1" t="n">
         <v>46040</v>
       </c>
-      <c r="Q1" s="2" t="n">
+      <c r="Q1" s="1" t="n">
         <v>46041</v>
       </c>
-      <c r="R1" s="2" t="n">
+      <c r="R1" s="1" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="2" t="n">
+      <c r="S1" s="1" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="2" t="n">
+      <c r="T1" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="2" t="n">
+      <c r="U1" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="2" t="n">
+      <c r="V1" s="1" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="2" t="n">
+      <c r="W1" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="2" t="n">
+      <c r="X1" s="1" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="2" t="n">
+      <c r="Y1" s="1" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="2" t="n">
+      <c r="Z1" s="1" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="2" t="n">
+      <c r="AA1" s="1" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="2" t="n">
+      <c r="AB1" s="1" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="2" t="n">
+      <c r="AC1" s="1" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="2" t="n">
+      <c r="AD1" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="2" t="n">
+      <c r="AE1" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="2" t="n">
+      <c r="AF1" s="1" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="2" t="n">
+      <c r="AG1" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="2" t="n">
+      <c r="AH1" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="2" t="n">
+      <c r="AI1" s="1" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="2" t="n">
+      <c r="AJ1" s="1" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="2" t="n">
+      <c r="AK1" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="2" t="n">
+      <c r="AL1" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="2" t="n">
+      <c r="AM1" s="1" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="2" t="n">
+      <c r="AN1" s="1" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="2" t="n">
+      <c r="AO1" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="2" t="n">
+      <c r="AP1" s="1" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="2" t="n">
+      <c r="AQ1" s="1" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="2" t="n">
+      <c r="AR1" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="2" t="n">
+      <c r="AS1" s="1" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="2" t="n">
+      <c r="AT1" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="2" t="n">
+      <c r="AU1" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="2" t="n">
+      <c r="AV1" s="1" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="2" t="n">
+      <c r="AW1" s="1" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="2" t="n">
+      <c r="AX1" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="2" t="n">
+      <c r="AY1" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="2" t="n">
+      <c r="AZ1" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="2" t="n">
+      <c r="BA1" s="1" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="2" t="n">
+      <c r="BB1" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="2" t="n">
+      <c r="BC1" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="2" t="n">
+      <c r="BD1" s="1" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="2" t="n">
+      <c r="BE1" s="1" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="2" t="n">
+      <c r="BF1" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="2" t="n">
+      <c r="BG1" s="1" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="2" t="n">
+      <c r="BH1" s="1" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="2" t="n">
+      <c r="BI1" s="1" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="2" t="n">
+      <c r="BJ1" s="1" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="2" t="n">
+      <c r="BK1" s="1" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="2" t="n">
+      <c r="BL1" s="1" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="2" t="n">
+      <c r="BM1" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="2" t="n">
+      <c r="BN1" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="2" t="n">
+      <c r="BO1" s="1" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="2" t="n">
+      <c r="BP1" s="1" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="2" t="n">
+      <c r="BQ1" s="1" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="2" t="n">
+      <c r="BR1" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="2" t="n">
+      <c r="BS1" s="1" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="2" t="n">
+      <c r="BT1" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="2" t="n">
+      <c r="BU1" s="1" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="2" t="n">
+      <c r="BV1" s="1" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="2" t="n">
+      <c r="BW1" s="1" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="2" t="n">
+      <c r="BX1" s="1" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="2" t="n">
+      <c r="BY1" s="1" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="2" t="n">
+      <c r="BZ1" s="1" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="2" t="n">
+      <c r="CA1" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="2" t="n">
+      <c r="CB1" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="2" t="n">
+      <c r="CC1" s="1" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="2" t="n">
+      <c r="CD1" s="1" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="2" t="n">
+      <c r="CE1" s="1" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="2" t="n">
+      <c r="CF1" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="2" t="n">
+      <c r="CG1" s="1" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="2" t="n">
+      <c r="CH1" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="2" t="n">
+      <c r="CI1" s="1" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="2" t="n">
+      <c r="CJ1" s="1" t="n">
         <v>46112</v>
       </c>
-      <c r="CK1" s="2" t="n">
+      <c r="CK1" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="CL1" s="2" t="n">
+      <c r="CL1" s="1" t="n">
         <v>46024</v>
       </c>
-      <c r="CM1" s="2" t="n">
+      <c r="CM1" s="1" t="n">
         <v>46025</v>
       </c>
-      <c r="CN1" s="2" t="n">
+      <c r="CN1" s="1" t="n">
         <v>46026</v>
       </c>
-      <c r="CO1" s="2" t="n">
+      <c r="CO1" s="1" t="n">
         <v>46027</v>
       </c>
-      <c r="CP1" s="2" t="n">
+      <c r="CP1" s="1" t="n">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="2" t="n">
+      <c r="CQ1" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="CR1" s="2" t="n">
+      <c r="CR1" s="1" t="n">
         <v>46114</v>
       </c>
-      <c r="CS1" s="2" t="n">
+      <c r="CS1" s="1" t="n">
         <v>46115</v>
       </c>
-      <c r="CT1" s="2" t="n">
+      <c r="CT1" s="1" t="n">
         <v>46116</v>
       </c>
-      <c r="CU1" s="2" t="n">
+      <c r="CU1" s="1" t="n">
         <v>46117</v>
       </c>
-      <c r="CV1" s="2" t="n">
+      <c r="CV1" s="1" t="n">
         <v>46118</v>
       </c>
-      <c r="CW1" s="2" t="n">
+      <c r="CW1" s="1" t="n">
         <v>46119</v>
       </c>
-      <c r="CX1" s="2" t="n">
+      <c r="CX1" s="1" t="n">
         <v>46120</v>
       </c>
-      <c r="CY1" s="2" t="n">
+      <c r="CY1" s="1" t="n">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="2" t="n">
+      <c r="CZ1" s="1" t="n">
         <v>46122</v>
       </c>
-      <c r="DA1" s="2" t="n">
+      <c r="DA1" s="1" t="n">
         <v>46123</v>
       </c>
-      <c r="DB1" s="2" t="n">
+      <c r="DB1" s="1" t="n">
         <v>46124</v>
       </c>
-      <c r="DC1" s="2" t="n">
+      <c r="DC1" s="1" t="n">
         <v>46125</v>
       </c>
-      <c r="DD1" s="2" t="n">
+      <c r="DD1" s="1" t="n">
         <v>46126</v>
       </c>
-      <c r="DE1" s="2" t="n">
+      <c r="DE1" s="1" t="n">
         <v>46127</v>
       </c>
-      <c r="DF1" s="2" t="n">
+      <c r="DF1" s="1" t="n">
         <v>46128</v>
       </c>
-      <c r="DG1" s="2" t="n">
+      <c r="DG1" s="1" t="n">
         <v>46129</v>
       </c>
-      <c r="DH1" s="2" t="n">
+      <c r="DH1" s="1" t="n">
         <v>46130</v>
       </c>
-      <c r="DI1" s="2" t="n">
+      <c r="DI1" s="1" t="n">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="2" t="n">
+      <c r="DJ1" s="1" t="n">
         <v>46132</v>
       </c>
-      <c r="DK1" s="2" t="n">
+      <c r="DK1" s="1" t="n">
         <v>46133</v>
       </c>
-      <c r="DL1" s="2" t="n">
+      <c r="DL1" s="1" t="n">
         <v>46134</v>
       </c>
-      <c r="DM1" s="2" t="n">
+      <c r="DM1" s="1" t="n">
         <v>46135</v>
       </c>
-      <c r="DN1" s="2" t="n">
+      <c r="DN1" s="1" t="n">
         <v>46136</v>
       </c>
-      <c r="DO1" s="2" t="n">
+      <c r="DO1" s="1" t="n">
         <v>46137</v>
       </c>
-      <c r="DP1" s="2" t="n">
+      <c r="DP1" s="1" t="n">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="2" t="n">
+      <c r="DQ1" s="1" t="n">
         <v>46139</v>
       </c>
-      <c r="DR1" s="2" t="n">
+      <c r="DR1" s="1" t="n">
         <v>46140</v>
       </c>
-      <c r="DS1" s="2" t="n">
+      <c r="DS1" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="DT1" s="2" t="n">
+      <c r="DT1" s="1" t="n">
         <v>46142</v>
       </c>
-      <c r="DU1" s="2" t="n">
+      <c r="DU1" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="DV1" s="2" t="n">
+      <c r="DV1" s="1" t="n">
         <v>46144</v>
       </c>
-      <c r="DW1" s="2" t="n">
+      <c r="DW1" s="1" t="n">
         <v>46145</v>
       </c>
-      <c r="DX1" s="2" t="n">
+      <c r="DX1" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="DY1" s="2" t="n">
+      <c r="DY1" s="1" t="n">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="2" t="n">
+      <c r="DZ1" s="1" t="n">
         <v>46148</v>
       </c>
-      <c r="EA1" s="2" t="n">
+      <c r="EA1" s="1" t="n">
         <v>46149</v>
       </c>
-      <c r="EB1" s="2" t="n">
+      <c r="EB1" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="EC1" s="2" t="n">
+      <c r="EC1" s="1" t="n">
         <v>46151</v>
       </c>
-      <c r="ED1" s="2" t="n">
+      <c r="ED1" s="1" t="n">
         <v>46152</v>
       </c>
-      <c r="EE1" s="2" t="n">
+      <c r="EE1" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="EF1" s="2" t="n">
+      <c r="EF1" s="1" t="n">
         <v>46154</v>
       </c>
-      <c r="EG1" s="2" t="n">
+      <c r="EG1" s="1" t="n">
         <v>46155</v>
       </c>
-      <c r="EH1" s="2" t="n">
+      <c r="EH1" s="1" t="n">
         <v>46156</v>
       </c>
-      <c r="EI1" s="2" t="n">
+      <c r="EI1" s="1" t="n">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="2" t="n">
+      <c r="EJ1" s="1" t="n">
         <v>46158</v>
       </c>
-      <c r="EK1" s="2" t="n">
+      <c r="EK1" s="1" t="n">
         <v>46159</v>
       </c>
-      <c r="EL1" s="2" t="n">
+      <c r="EL1" s="1" t="n">
         <v>46160</v>
       </c>
-      <c r="EM1" s="2" t="n">
+      <c r="EM1" s="1" t="n">
         <v>46161</v>
       </c>
-      <c r="EN1" s="2" t="n">
+      <c r="EN1" s="1" t="n">
         <v>46162</v>
       </c>
-      <c r="EO1" s="2" t="n">
+      <c r="EO1" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="EP1" s="2" t="n">
+      <c r="EP1" s="1" t="n">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="2" t="n">
+      <c r="EQ1" s="1" t="n">
         <v>46165</v>
       </c>
-      <c r="ER1" s="2" t="n">
+      <c r="ER1" s="1" t="n">
         <v>46166</v>
       </c>
-      <c r="ES1" s="2" t="n">
+      <c r="ES1" s="1" t="n">
         <v>46167</v>
       </c>
-      <c r="ET1" s="2" t="n">
+      <c r="ET1" s="1" t="n">
         <v>46168</v>
       </c>
-      <c r="EU1" s="2" t="n">
+      <c r="EU1" s="1" t="n">
         <v>46169</v>
       </c>
-      <c r="EV1" s="2" t="n">
+      <c r="EV1" s="1" t="n">
         <v>46170</v>
       </c>
-      <c r="EW1" s="2" t="n">
+      <c r="EW1" s="1" t="n">
         <v>46171</v>
       </c>
-      <c r="EX1" s="2" t="n">
+      <c r="EX1" s="1" t="n">
         <v>46172</v>
       </c>
-      <c r="EY1" s="2" t="n">
+      <c r="EY1" s="1" t="n">
         <v>46173</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Site Manager</t>
+          <t>Supervisor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jose Gomez Ch</t>
+          <t>Aldair Hernandez</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>E786</t>
-        </is>
-      </c>
-      <c r="AL2" s="3" t="inlineStr">
+          <t>K321</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AN2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
+      <c r="AP2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fuel Attendant</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Elver Gonzales</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>KL569</t>
+      <c r="AQ2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="CK2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
popup colision funcional ahora el codigo se debe de someter a pruebas
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -926,64 +926,74 @@
           <t>K321</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AL2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AM2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AL2" s="2" t="inlineStr">
+      <c r="AQ2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AS2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AT2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AU2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AP2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AQ2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AR2" s="2" t="inlineStr">
+      <c r="AW2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AX2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="AT2" s="2" t="inlineStr">
+      <c r="AY2" s="2" t="inlineStr">
         <is>
           <t>ON NS</t>
         </is>
       </c>
-      <c r="CK2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>ON NS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correcion de flasheo al asignar el usuario ya no se mueve la pantalla
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -27,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +47,12 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,11 +66,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY2"/>
+  <dimension ref="A1:EZ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -909,6 +918,9 @@
       <c r="EY1" s="1" t="n">
         <v>46173</v>
       </c>
+      <c r="EZ1" s="4" t="n">
+        <v>46022</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -926,6 +938,36 @@
           <t>K321</t>
         </is>
       </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AJ2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AK2" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="AL2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
@@ -941,59 +983,14 @@
           <t>ON</t>
         </is>
       </c>
-      <c r="AO2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AP2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AQ2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AS2" s="3" t="inlineStr">
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="AT2" s="3" t="inlineStr">
+      <c r="AP2" s="3" t="inlineStr">
         <is>
           <t>ON</t>
-        </is>
-      </c>
-      <c r="AU2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AW2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AX2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AY2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BE2" s="2" t="inlineStr">
-        <is>
-          <t>ON NS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh de colores funcional pero en fase de testing
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -15,9 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -28,30 +27,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,13 +47,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,532 +443,477 @@
           <t>BADGE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" s="2" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" s="2" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" s="2" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" s="2" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" s="2" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="2" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" s="2" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" s="2" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" s="2" t="n">
         <v>46039</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" s="2" t="n">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" s="2" t="n">
         <v>46041</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" s="2" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" s="2" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" s="2" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" s="2" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" s="2" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" s="2" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" s="2" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" s="2" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" s="2" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" s="2" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" s="2" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" s="2" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" s="2" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" s="2" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" s="2" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" s="2" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" s="2" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" s="2" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" s="2" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" s="2" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" s="2" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" s="2" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" s="2" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" s="2" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" s="2" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" s="2" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" s="2" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" s="2" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1" t="n">
+      <c r="AW1" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1" t="n">
+      <c r="AX1" s="2" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1" t="n">
+      <c r="AY1" s="2" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1" t="n">
+      <c r="AZ1" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1" t="n">
+      <c r="BA1" s="2" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1" t="n">
+      <c r="BB1" s="2" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1" t="n">
+      <c r="BC1" s="2" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1" t="n">
+      <c r="BD1" s="2" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1" t="n">
+      <c r="BE1" s="2" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1" t="n">
+      <c r="BF1" s="2" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1" t="n">
+      <c r="BG1" s="2" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1" t="n">
+      <c r="BH1" s="2" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1" t="n">
+      <c r="BI1" s="2" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1" t="n">
+      <c r="BJ1" s="2" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1" t="n">
+      <c r="BK1" s="2" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1" t="n">
+      <c r="BL1" s="2" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1" t="n">
+      <c r="BM1" s="2" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1" t="n">
+      <c r="BN1" s="2" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1" t="n">
+      <c r="BO1" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1" t="n">
+      <c r="BP1" s="2" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1" t="n">
+      <c r="BQ1" s="2" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1" t="n">
+      <c r="BR1" s="2" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1" t="n">
+      <c r="BS1" s="2" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1" t="n">
+      <c r="BT1" s="2" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1" t="n">
+      <c r="BU1" s="2" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1" t="n">
+      <c r="BV1" s="2" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1" t="n">
+      <c r="BW1" s="2" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1" t="n">
+      <c r="BX1" s="2" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1" t="n">
+      <c r="BY1" s="2" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1" t="n">
+      <c r="BZ1" s="2" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1" t="n">
+      <c r="CA1" s="2" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1" t="n">
+      <c r="CB1" s="2" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1" t="n">
+      <c r="CC1" s="2" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1" t="n">
+      <c r="CD1" s="2" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1" t="n">
+      <c r="CE1" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1" t="n">
+      <c r="CF1" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1" t="n">
+      <c r="CG1" s="2" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1" t="n">
+      <c r="CH1" s="2" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1" t="n">
+      <c r="CI1" s="2" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1" t="n">
+      <c r="CJ1" s="2" t="n">
         <v>46112</v>
       </c>
-      <c r="CK1" s="1" t="n">
+      <c r="CK1" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="CL1" s="1" t="n">
+      <c r="CL1" s="2" t="n">
         <v>46024</v>
       </c>
-      <c r="CM1" s="1" t="n">
+      <c r="CM1" s="2" t="n">
         <v>46025</v>
       </c>
-      <c r="CN1" s="1" t="n">
+      <c r="CN1" s="2" t="n">
         <v>46026</v>
       </c>
-      <c r="CO1" s="1" t="n">
+      <c r="CO1" s="2" t="n">
         <v>46027</v>
       </c>
-      <c r="CP1" s="1" t="n">
+      <c r="CP1" s="2" t="n">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="1" t="n">
+      <c r="CQ1" s="2" t="n">
         <v>46113</v>
       </c>
-      <c r="CR1" s="1" t="n">
+      <c r="CR1" s="2" t="n">
         <v>46114</v>
       </c>
-      <c r="CS1" s="1" t="n">
+      <c r="CS1" s="2" t="n">
         <v>46115</v>
       </c>
-      <c r="CT1" s="1" t="n">
+      <c r="CT1" s="2" t="n">
         <v>46116</v>
       </c>
-      <c r="CU1" s="1" t="n">
+      <c r="CU1" s="2" t="n">
         <v>46117</v>
       </c>
-      <c r="CV1" s="1" t="n">
+      <c r="CV1" s="2" t="n">
         <v>46118</v>
       </c>
-      <c r="CW1" s="1" t="n">
+      <c r="CW1" s="2" t="n">
         <v>46119</v>
       </c>
-      <c r="CX1" s="1" t="n">
+      <c r="CX1" s="2" t="n">
         <v>46120</v>
       </c>
-      <c r="CY1" s="1" t="n">
+      <c r="CY1" s="2" t="n">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="1" t="n">
+      <c r="CZ1" s="2" t="n">
         <v>46122</v>
       </c>
-      <c r="DA1" s="1" t="n">
+      <c r="DA1" s="2" t="n">
         <v>46123</v>
       </c>
-      <c r="DB1" s="1" t="n">
+      <c r="DB1" s="2" t="n">
         <v>46124</v>
       </c>
-      <c r="DC1" s="1" t="n">
+      <c r="DC1" s="2" t="n">
         <v>46125</v>
       </c>
-      <c r="DD1" s="1" t="n">
+      <c r="DD1" s="2" t="n">
         <v>46126</v>
       </c>
-      <c r="DE1" s="1" t="n">
+      <c r="DE1" s="2" t="n">
         <v>46127</v>
       </c>
-      <c r="DF1" s="1" t="n">
+      <c r="DF1" s="2" t="n">
         <v>46128</v>
       </c>
-      <c r="DG1" s="1" t="n">
+      <c r="DG1" s="2" t="n">
         <v>46129</v>
       </c>
-      <c r="DH1" s="1" t="n">
+      <c r="DH1" s="2" t="n">
         <v>46130</v>
       </c>
-      <c r="DI1" s="1" t="n">
+      <c r="DI1" s="2" t="n">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="1" t="n">
+      <c r="DJ1" s="2" t="n">
         <v>46132</v>
       </c>
-      <c r="DK1" s="1" t="n">
+      <c r="DK1" s="2" t="n">
         <v>46133</v>
       </c>
-      <c r="DL1" s="1" t="n">
+      <c r="DL1" s="2" t="n">
         <v>46134</v>
       </c>
-      <c r="DM1" s="1" t="n">
+      <c r="DM1" s="2" t="n">
         <v>46135</v>
       </c>
-      <c r="DN1" s="1" t="n">
+      <c r="DN1" s="2" t="n">
         <v>46136</v>
       </c>
-      <c r="DO1" s="1" t="n">
+      <c r="DO1" s="2" t="n">
         <v>46137</v>
       </c>
-      <c r="DP1" s="1" t="n">
+      <c r="DP1" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="1" t="n">
+      <c r="DQ1" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="DR1" s="1" t="n">
+      <c r="DR1" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="DS1" s="1" t="n">
+      <c r="DS1" s="2" t="n">
         <v>46141</v>
       </c>
-      <c r="DT1" s="1" t="n">
+      <c r="DT1" s="2" t="n">
         <v>46142</v>
       </c>
-      <c r="DU1" s="1" t="n">
+      <c r="DU1" s="2" t="n">
         <v>46143</v>
       </c>
-      <c r="DV1" s="1" t="n">
+      <c r="DV1" s="2" t="n">
         <v>46144</v>
       </c>
-      <c r="DW1" s="1" t="n">
+      <c r="DW1" s="2" t="n">
         <v>46145</v>
       </c>
-      <c r="DX1" s="1" t="n">
+      <c r="DX1" s="2" t="n">
         <v>46146</v>
       </c>
-      <c r="DY1" s="1" t="n">
+      <c r="DY1" s="2" t="n">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="1" t="n">
+      <c r="DZ1" s="2" t="n">
         <v>46148</v>
       </c>
-      <c r="EA1" s="1" t="n">
+      <c r="EA1" s="2" t="n">
         <v>46149</v>
       </c>
-      <c r="EB1" s="1" t="n">
+      <c r="EB1" s="2" t="n">
         <v>46150</v>
       </c>
-      <c r="EC1" s="1" t="n">
+      <c r="EC1" s="2" t="n">
         <v>46151</v>
       </c>
-      <c r="ED1" s="1" t="n">
+      <c r="ED1" s="2" t="n">
         <v>46152</v>
       </c>
-      <c r="EE1" s="1" t="n">
+      <c r="EE1" s="2" t="n">
         <v>46153</v>
       </c>
-      <c r="EF1" s="1" t="n">
+      <c r="EF1" s="2" t="n">
         <v>46154</v>
       </c>
-      <c r="EG1" s="1" t="n">
+      <c r="EG1" s="2" t="n">
         <v>46155</v>
       </c>
-      <c r="EH1" s="1" t="n">
+      <c r="EH1" s="2" t="n">
         <v>46156</v>
       </c>
-      <c r="EI1" s="1" t="n">
+      <c r="EI1" s="2" t="n">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="1" t="n">
+      <c r="EJ1" s="2" t="n">
         <v>46158</v>
       </c>
-      <c r="EK1" s="1" t="n">
+      <c r="EK1" s="2" t="n">
         <v>46159</v>
       </c>
-      <c r="EL1" s="1" t="n">
+      <c r="EL1" s="2" t="n">
         <v>46160</v>
       </c>
-      <c r="EM1" s="1" t="n">
+      <c r="EM1" s="2" t="n">
         <v>46161</v>
       </c>
-      <c r="EN1" s="1" t="n">
+      <c r="EN1" s="2" t="n">
         <v>46162</v>
       </c>
-      <c r="EO1" s="1" t="n">
+      <c r="EO1" s="2" t="n">
         <v>46163</v>
       </c>
-      <c r="EP1" s="1" t="n">
+      <c r="EP1" s="2" t="n">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="1" t="n">
+      <c r="EQ1" s="2" t="n">
         <v>46165</v>
       </c>
-      <c r="ER1" s="1" t="n">
+      <c r="ER1" s="2" t="n">
         <v>46166</v>
       </c>
-      <c r="ES1" s="1" t="n">
+      <c r="ES1" s="2" t="n">
         <v>46167</v>
       </c>
-      <c r="ET1" s="1" t="n">
+      <c r="ET1" s="2" t="n">
         <v>46168</v>
       </c>
-      <c r="EU1" s="1" t="n">
+      <c r="EU1" s="2" t="n">
         <v>46169</v>
       </c>
-      <c r="EV1" s="1" t="n">
+      <c r="EV1" s="2" t="n">
         <v>46170</v>
       </c>
-      <c r="EW1" s="1" t="n">
+      <c r="EW1" s="2" t="n">
         <v>46171</v>
       </c>
-      <c r="EX1" s="1" t="n">
+      <c r="EX1" s="2" t="n">
         <v>46172</v>
       </c>
-      <c r="EY1" s="1" t="n">
+      <c r="EY1" s="2" t="n">
         <v>46173</v>
       </c>
-      <c r="EZ1" s="4" t="n">
+      <c r="EZ1" s="2" t="n">
         <v>46022</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Supervisor</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Aldair Hernandez</t>
+          <t>Carlos Gomez</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>K321</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AJ2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AK2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AL2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AM2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AP2" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
+          <t>N536</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
esta no se puede eliminar location y role atados a usuarios
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -27,12 +27,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,10 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EZ2"/>
+  <dimension ref="A1:EZ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -917,6 +938,100 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jose Gomez</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>L698</t>
+        </is>
+      </c>
+      <c r="AM3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AN3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AO3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AP3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AQ3" s="5" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AR3" s="5" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="AS3" s="5" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="BG3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BH3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BI3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BJ3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="BK3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Juan Gonzales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>L968</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
funciona la asignacion de ON y ONs dia dia anterior pero debe de hacer correcion
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,56 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1+D CRUD\inboundoutbound\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46495E83-4F7B-47B0-96A7-75A5D4D76F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>TEAM</t>
+  </si>
+  <si>
+    <t>ROLE</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>BADGE</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -65,86 +75,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -432,604 +379,481 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:EZ4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:EZ1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
+    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ROLE</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>NAME</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>BADGE</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="n">
+    <row r="1" spans="1:156" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1">
         <v>46029</v>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="F1" s="1">
         <v>46030</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="1">
         <v>46031</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="H1" s="1">
         <v>46032</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="I1" s="1">
         <v>46033</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="1">
         <v>46034</v>
       </c>
-      <c r="K1" s="2" t="n">
+      <c r="K1" s="1">
         <v>46035</v>
       </c>
-      <c r="L1" s="2" t="n">
+      <c r="L1" s="1">
         <v>46036</v>
       </c>
-      <c r="M1" s="2" t="n">
+      <c r="M1" s="1">
         <v>46037</v>
       </c>
-      <c r="N1" s="2" t="n">
+      <c r="N1" s="1">
         <v>46038</v>
       </c>
-      <c r="O1" s="2" t="n">
+      <c r="O1" s="1">
         <v>46039</v>
       </c>
-      <c r="P1" s="2" t="n">
+      <c r="P1" s="1">
         <v>46040</v>
       </c>
-      <c r="Q1" s="2" t="n">
+      <c r="Q1" s="1">
         <v>46041</v>
       </c>
-      <c r="R1" s="2" t="n">
+      <c r="R1" s="1">
         <v>46042</v>
       </c>
-      <c r="S1" s="2" t="n">
+      <c r="S1" s="1">
         <v>46043</v>
       </c>
-      <c r="T1" s="2" t="n">
+      <c r="T1" s="1">
         <v>46044</v>
       </c>
-      <c r="U1" s="2" t="n">
+      <c r="U1" s="1">
         <v>46045</v>
       </c>
-      <c r="V1" s="2" t="n">
+      <c r="V1" s="1">
         <v>46046</v>
       </c>
-      <c r="W1" s="2" t="n">
+      <c r="W1" s="1">
         <v>46047</v>
       </c>
-      <c r="X1" s="2" t="n">
+      <c r="X1" s="1">
         <v>46048</v>
       </c>
-      <c r="Y1" s="2" t="n">
+      <c r="Y1" s="1">
         <v>46049</v>
       </c>
-      <c r="Z1" s="2" t="n">
+      <c r="Z1" s="1">
         <v>46050</v>
       </c>
-      <c r="AA1" s="2" t="n">
+      <c r="AA1" s="1">
         <v>46051</v>
       </c>
-      <c r="AB1" s="2" t="n">
+      <c r="AB1" s="1">
         <v>46052</v>
       </c>
-      <c r="AC1" s="2" t="n">
+      <c r="AC1" s="1">
         <v>46053</v>
       </c>
-      <c r="AD1" s="2" t="n">
+      <c r="AD1" s="1">
         <v>46054</v>
       </c>
-      <c r="AE1" s="2" t="n">
+      <c r="AE1" s="1">
         <v>46055</v>
       </c>
-      <c r="AF1" s="2" t="n">
+      <c r="AF1" s="1">
         <v>46056</v>
       </c>
-      <c r="AG1" s="2" t="n">
+      <c r="AG1" s="1">
         <v>46057</v>
       </c>
-      <c r="AH1" s="2" t="n">
+      <c r="AH1" s="1">
         <v>46058</v>
       </c>
-      <c r="AI1" s="2" t="n">
+      <c r="AI1" s="1">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="2" t="n">
+      <c r="AJ1" s="1">
         <v>46060</v>
       </c>
-      <c r="AK1" s="2" t="n">
+      <c r="AK1" s="1">
         <v>46061</v>
       </c>
-      <c r="AL1" s="2" t="n">
+      <c r="AL1" s="1">
         <v>46062</v>
       </c>
-      <c r="AM1" s="2" t="n">
+      <c r="AM1" s="1">
         <v>46063</v>
       </c>
-      <c r="AN1" s="2" t="n">
+      <c r="AN1" s="1">
         <v>46064</v>
       </c>
-      <c r="AO1" s="2" t="n">
+      <c r="AO1" s="1">
         <v>46065</v>
       </c>
-      <c r="AP1" s="2" t="n">
+      <c r="AP1" s="1">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="2" t="n">
+      <c r="AQ1" s="1">
         <v>46067</v>
       </c>
-      <c r="AR1" s="2" t="n">
+      <c r="AR1" s="1">
         <v>46068</v>
       </c>
-      <c r="AS1" s="2" t="n">
+      <c r="AS1" s="1">
         <v>46069</v>
       </c>
-      <c r="AT1" s="2" t="n">
+      <c r="AT1" s="1">
         <v>46070</v>
       </c>
-      <c r="AU1" s="2" t="n">
+      <c r="AU1" s="1">
         <v>46071</v>
       </c>
-      <c r="AV1" s="2" t="n">
+      <c r="AV1" s="1">
         <v>46072</v>
       </c>
-      <c r="AW1" s="2" t="n">
+      <c r="AW1" s="1">
         <v>46073</v>
       </c>
-      <c r="AX1" s="2" t="n">
+      <c r="AX1" s="1">
         <v>46074</v>
       </c>
-      <c r="AY1" s="2" t="n">
+      <c r="AY1" s="1">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="2" t="n">
+      <c r="AZ1" s="1">
         <v>46076</v>
       </c>
-      <c r="BA1" s="2" t="n">
+      <c r="BA1" s="1">
         <v>46077</v>
       </c>
-      <c r="BB1" s="2" t="n">
+      <c r="BB1" s="1">
         <v>46078</v>
       </c>
-      <c r="BC1" s="2" t="n">
+      <c r="BC1" s="1">
         <v>46079</v>
       </c>
-      <c r="BD1" s="2" t="n">
+      <c r="BD1" s="1">
         <v>46080</v>
       </c>
-      <c r="BE1" s="2" t="n">
+      <c r="BE1" s="1">
         <v>46081</v>
       </c>
-      <c r="BF1" s="2" t="n">
+      <c r="BF1" s="1">
         <v>46082</v>
       </c>
-      <c r="BG1" s="2" t="n">
+      <c r="BG1" s="1">
         <v>46083</v>
       </c>
-      <c r="BH1" s="2" t="n">
+      <c r="BH1" s="1">
         <v>46084</v>
       </c>
-      <c r="BI1" s="2" t="n">
+      <c r="BI1" s="1">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="2" t="n">
+      <c r="BJ1" s="1">
         <v>46086</v>
       </c>
-      <c r="BK1" s="2" t="n">
+      <c r="BK1" s="1">
         <v>46087</v>
       </c>
-      <c r="BL1" s="2" t="n">
+      <c r="BL1" s="1">
         <v>46088</v>
       </c>
-      <c r="BM1" s="2" t="n">
+      <c r="BM1" s="1">
         <v>46089</v>
       </c>
-      <c r="BN1" s="2" t="n">
+      <c r="BN1" s="1">
         <v>46090</v>
       </c>
-      <c r="BO1" s="2" t="n">
+      <c r="BO1" s="1">
         <v>46091</v>
       </c>
-      <c r="BP1" s="2" t="n">
+      <c r="BP1" s="1">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="2" t="n">
+      <c r="BQ1" s="1">
         <v>46093</v>
       </c>
-      <c r="BR1" s="2" t="n">
+      <c r="BR1" s="1">
         <v>46094</v>
       </c>
-      <c r="BS1" s="2" t="n">
+      <c r="BS1" s="1">
         <v>46095</v>
       </c>
-      <c r="BT1" s="2" t="n">
+      <c r="BT1" s="1">
         <v>46096</v>
       </c>
-      <c r="BU1" s="2" t="n">
+      <c r="BU1" s="1">
         <v>46097</v>
       </c>
-      <c r="BV1" s="2" t="n">
+      <c r="BV1" s="1">
         <v>46098</v>
       </c>
-      <c r="BW1" s="2" t="n">
+      <c r="BW1" s="1">
         <v>46099</v>
       </c>
-      <c r="BX1" s="2" t="n">
+      <c r="BX1" s="1">
         <v>46100</v>
       </c>
-      <c r="BY1" s="2" t="n">
+      <c r="BY1" s="1">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="2" t="n">
+      <c r="BZ1" s="1">
         <v>46102</v>
       </c>
-      <c r="CA1" s="2" t="n">
+      <c r="CA1" s="1">
         <v>46103</v>
       </c>
-      <c r="CB1" s="2" t="n">
+      <c r="CB1" s="1">
         <v>46104</v>
       </c>
-      <c r="CC1" s="2" t="n">
+      <c r="CC1" s="1">
         <v>46105</v>
       </c>
-      <c r="CD1" s="2" t="n">
+      <c r="CD1" s="1">
         <v>46106</v>
       </c>
-      <c r="CE1" s="2" t="n">
+      <c r="CE1" s="1">
         <v>46107</v>
       </c>
-      <c r="CF1" s="2" t="n">
+      <c r="CF1" s="1">
         <v>46108</v>
       </c>
-      <c r="CG1" s="2" t="n">
+      <c r="CG1" s="1">
         <v>46109</v>
       </c>
-      <c r="CH1" s="2" t="n">
+      <c r="CH1" s="1">
         <v>46110</v>
       </c>
-      <c r="CI1" s="2" t="n">
+      <c r="CI1" s="1">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="2" t="n">
+      <c r="CJ1" s="1">
         <v>46112</v>
       </c>
-      <c r="CK1" s="2" t="n">
+      <c r="CK1" s="1">
         <v>46023</v>
       </c>
-      <c r="CL1" s="2" t="n">
+      <c r="CL1" s="1">
         <v>46024</v>
       </c>
-      <c r="CM1" s="2" t="n">
+      <c r="CM1" s="1">
         <v>46025</v>
       </c>
-      <c r="CN1" s="2" t="n">
+      <c r="CN1" s="1">
         <v>46026</v>
       </c>
-      <c r="CO1" s="2" t="n">
+      <c r="CO1" s="1">
         <v>46027</v>
       </c>
-      <c r="CP1" s="2" t="n">
+      <c r="CP1" s="1">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="2" t="n">
+      <c r="CQ1" s="1">
         <v>46113</v>
       </c>
-      <c r="CR1" s="2" t="n">
+      <c r="CR1" s="1">
         <v>46114</v>
       </c>
-      <c r="CS1" s="2" t="n">
+      <c r="CS1" s="1">
         <v>46115</v>
       </c>
-      <c r="CT1" s="2" t="n">
+      <c r="CT1" s="1">
         <v>46116</v>
       </c>
-      <c r="CU1" s="2" t="n">
+      <c r="CU1" s="1">
         <v>46117</v>
       </c>
-      <c r="CV1" s="2" t="n">
+      <c r="CV1" s="1">
         <v>46118</v>
       </c>
-      <c r="CW1" s="2" t="n">
+      <c r="CW1" s="1">
         <v>46119</v>
       </c>
-      <c r="CX1" s="2" t="n">
+      <c r="CX1" s="1">
         <v>46120</v>
       </c>
-      <c r="CY1" s="2" t="n">
+      <c r="CY1" s="1">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="2" t="n">
+      <c r="CZ1" s="1">
         <v>46122</v>
       </c>
-      <c r="DA1" s="2" t="n">
+      <c r="DA1" s="1">
         <v>46123</v>
       </c>
-      <c r="DB1" s="2" t="n">
+      <c r="DB1" s="1">
         <v>46124</v>
       </c>
-      <c r="DC1" s="2" t="n">
+      <c r="DC1" s="1">
         <v>46125</v>
       </c>
-      <c r="DD1" s="2" t="n">
+      <c r="DD1" s="1">
         <v>46126</v>
       </c>
-      <c r="DE1" s="2" t="n">
+      <c r="DE1" s="1">
         <v>46127</v>
       </c>
-      <c r="DF1" s="2" t="n">
+      <c r="DF1" s="1">
         <v>46128</v>
       </c>
-      <c r="DG1" s="2" t="n">
+      <c r="DG1" s="1">
         <v>46129</v>
       </c>
-      <c r="DH1" s="2" t="n">
+      <c r="DH1" s="1">
         <v>46130</v>
       </c>
-      <c r="DI1" s="2" t="n">
+      <c r="DI1" s="1">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="2" t="n">
+      <c r="DJ1" s="1">
         <v>46132</v>
       </c>
-      <c r="DK1" s="2" t="n">
+      <c r="DK1" s="1">
         <v>46133</v>
       </c>
-      <c r="DL1" s="2" t="n">
+      <c r="DL1" s="1">
         <v>46134</v>
       </c>
-      <c r="DM1" s="2" t="n">
+      <c r="DM1" s="1">
         <v>46135</v>
       </c>
-      <c r="DN1" s="2" t="n">
+      <c r="DN1" s="1">
         <v>46136</v>
       </c>
-      <c r="DO1" s="2" t="n">
+      <c r="DO1" s="1">
         <v>46137</v>
       </c>
-      <c r="DP1" s="2" t="n">
+      <c r="DP1" s="1">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="2" t="n">
+      <c r="DQ1" s="1">
         <v>46139</v>
       </c>
-      <c r="DR1" s="2" t="n">
+      <c r="DR1" s="1">
         <v>46140</v>
       </c>
-      <c r="DS1" s="2" t="n">
+      <c r="DS1" s="1">
         <v>46141</v>
       </c>
-      <c r="DT1" s="2" t="n">
+      <c r="DT1" s="1">
         <v>46142</v>
       </c>
-      <c r="DU1" s="2" t="n">
+      <c r="DU1" s="1">
         <v>46143</v>
       </c>
-      <c r="DV1" s="2" t="n">
+      <c r="DV1" s="1">
         <v>46144</v>
       </c>
-      <c r="DW1" s="2" t="n">
+      <c r="DW1" s="1">
         <v>46145</v>
       </c>
-      <c r="DX1" s="2" t="n">
+      <c r="DX1" s="1">
         <v>46146</v>
       </c>
-      <c r="DY1" s="2" t="n">
+      <c r="DY1" s="1">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="2" t="n">
+      <c r="DZ1" s="1">
         <v>46148</v>
       </c>
-      <c r="EA1" s="2" t="n">
+      <c r="EA1" s="1">
         <v>46149</v>
       </c>
-      <c r="EB1" s="2" t="n">
+      <c r="EB1" s="1">
         <v>46150</v>
       </c>
-      <c r="EC1" s="2" t="n">
+      <c r="EC1" s="1">
         <v>46151</v>
       </c>
-      <c r="ED1" s="2" t="n">
+      <c r="ED1" s="1">
         <v>46152</v>
       </c>
-      <c r="EE1" s="2" t="n">
+      <c r="EE1" s="1">
         <v>46153</v>
       </c>
-      <c r="EF1" s="2" t="n">
+      <c r="EF1" s="1">
         <v>46154</v>
       </c>
-      <c r="EG1" s="2" t="n">
+      <c r="EG1" s="1">
         <v>46155</v>
       </c>
-      <c r="EH1" s="2" t="n">
+      <c r="EH1" s="1">
         <v>46156</v>
       </c>
-      <c r="EI1" s="2" t="n">
+      <c r="EI1" s="1">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="2" t="n">
+      <c r="EJ1" s="1">
         <v>46158</v>
       </c>
-      <c r="EK1" s="2" t="n">
+      <c r="EK1" s="1">
         <v>46159</v>
       </c>
-      <c r="EL1" s="2" t="n">
+      <c r="EL1" s="1">
         <v>46160</v>
       </c>
-      <c r="EM1" s="2" t="n">
+      <c r="EM1" s="1">
         <v>46161</v>
       </c>
-      <c r="EN1" s="2" t="n">
+      <c r="EN1" s="1">
         <v>46162</v>
       </c>
-      <c r="EO1" s="2" t="n">
+      <c r="EO1" s="1">
         <v>46163</v>
       </c>
-      <c r="EP1" s="2" t="n">
+      <c r="EP1" s="1">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="2" t="n">
+      <c r="EQ1" s="1">
         <v>46165</v>
       </c>
-      <c r="ER1" s="2" t="n">
+      <c r="ER1" s="1">
         <v>46166</v>
       </c>
-      <c r="ES1" s="2" t="n">
+      <c r="ES1" s="1">
         <v>46167</v>
       </c>
-      <c r="ET1" s="2" t="n">
+      <c r="ET1" s="1">
         <v>46168</v>
       </c>
-      <c r="EU1" s="2" t="n">
+      <c r="EU1" s="1">
         <v>46169</v>
       </c>
-      <c r="EV1" s="2" t="n">
+      <c r="EV1" s="1">
         <v>46170</v>
       </c>
-      <c r="EW1" s="2" t="n">
+      <c r="EW1" s="1">
         <v>46171</v>
       </c>
-      <c r="EX1" s="2" t="n">
+      <c r="EX1" s="1">
         <v>46172</v>
       </c>
-      <c r="EY1" s="2" t="n">
+      <c r="EY1" s="1">
         <v>46173</v>
       </c>
-      <c r="EZ1" s="2" t="n">
+      <c r="EZ1" s="1">
         <v>46022</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Carlos Gomez</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N536</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Data Analyst</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Jose Gomez</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>L698</t>
-        </is>
-      </c>
-      <c r="AM3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AN3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AO3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AP3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="AQ3" s="5" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AR3" s="5" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="AS3" s="5" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="BG3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BH3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BI3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BJ3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="BK3" s="3" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Juan Gonzales</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>L968</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Error de Atributo Funcion Faltante Fixed
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -42,8 +42,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFAA7F"/>
+        <bgColor rgb="00FFAA7F"/>
       </patternFill>
     </fill>
     <fill>
@@ -145,6 +145,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ShiftType</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="CN2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="CO2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+    <comment ref="CP2" authorId="0" shapeId="0">
+      <text>
+        <t>00:00-00:00</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -923,7 +953,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Supervisor</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -933,81 +963,77 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>L632</t>
+          <t>L639</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>ON NS</t>
+        </is>
+      </c>
+      <c r="CK2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="CK2" s="2" t="inlineStr">
+      <c r="CL2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="CL2" s="2" t="inlineStr">
+      <c r="CM2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="CM2" s="2" t="inlineStr">
+      <c r="CN2" s="3" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="CO2" s="3" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="CP2" s="3" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="EZ2" s="2" t="inlineStr">
         <is>
           <t>ON</t>
-        </is>
-      </c>
-      <c r="CN2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CO2" s="3" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="CP2" s="3" t="inlineStr">
-        <is>
-          <t>OFF</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
esta funcional la opcion de crear work days que no requieran tranasporte
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,56 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1+D CRUD\inboundoutbound\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B2275E-1CEF-447C-A419-71F82033294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>TEAM</t>
+  </si>
+  <si>
+    <t>ROLE</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>BADGE</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFAA7F"/>
-        <bgColor rgb="00FFAA7F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -65,116 +75,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>ShiftType</author>
-  </authors>
-  <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="CN2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="CO2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-    <comment ref="CP2" authorId="0" shapeId="0">
-      <text>
-        <t>00:00-00:00</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -461,579 +379,484 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:EZ2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:EZ1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
+    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ROLE</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>NAME</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>BADGE</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="n">
+    <row r="1" spans="1:156" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1">
         <v>46029</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" s="1">
         <v>46030</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" s="1">
         <v>46031</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" s="1">
         <v>46032</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" s="1">
         <v>46033</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" s="1">
         <v>46034</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="1">
         <v>46035</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" s="1">
         <v>46036</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" s="1">
         <v>46037</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" s="1">
         <v>46038</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" s="1">
         <v>46039</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" s="1">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" s="1">
         <v>46041</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" s="1">
         <v>46042</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" s="1">
         <v>46043</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" s="1">
         <v>46044</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" s="1">
         <v>46045</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" s="1">
         <v>46046</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" s="1">
         <v>46047</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" s="1">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" s="1">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" s="1">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" s="1">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" s="1">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" s="1">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" s="1">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" s="1">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" s="1">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" s="1">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" s="1">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" s="1">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" s="1">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" s="1">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" s="1">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" s="1">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" s="1">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" s="1">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" s="1">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" s="1">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" s="1">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" s="1">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" s="1">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" s="1">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" s="1">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1" t="n">
+      <c r="AW1" s="1">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1" t="n">
+      <c r="AX1" s="1">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1" t="n">
+      <c r="AY1" s="1">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1" t="n">
+      <c r="AZ1" s="1">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1" t="n">
+      <c r="BA1" s="1">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1" t="n">
+      <c r="BB1" s="1">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1" t="n">
+      <c r="BC1" s="1">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1" t="n">
+      <c r="BD1" s="1">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1" t="n">
+      <c r="BE1" s="1">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1" t="n">
+      <c r="BF1" s="1">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1" t="n">
+      <c r="BG1" s="1">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1" t="n">
+      <c r="BH1" s="1">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1" t="n">
+      <c r="BI1" s="1">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1" t="n">
+      <c r="BJ1" s="1">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1" t="n">
+      <c r="BK1" s="1">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1" t="n">
+      <c r="BL1" s="1">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1" t="n">
+      <c r="BM1" s="1">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1" t="n">
+      <c r="BN1" s="1">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1" t="n">
+      <c r="BO1" s="1">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1" t="n">
+      <c r="BP1" s="1">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1" t="n">
+      <c r="BQ1" s="1">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1" t="n">
+      <c r="BR1" s="1">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1" t="n">
+      <c r="BS1" s="1">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1" t="n">
+      <c r="BT1" s="1">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1" t="n">
+      <c r="BU1" s="1">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1" t="n">
+      <c r="BV1" s="1">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1" t="n">
+      <c r="BW1" s="1">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1" t="n">
+      <c r="BX1" s="1">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1" t="n">
+      <c r="BY1" s="1">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1" t="n">
+      <c r="BZ1" s="1">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1" t="n">
+      <c r="CA1" s="1">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1" t="n">
+      <c r="CB1" s="1">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1" t="n">
+      <c r="CC1" s="1">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1" t="n">
+      <c r="CD1" s="1">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1" t="n">
+      <c r="CE1" s="1">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1" t="n">
+      <c r="CF1" s="1">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1" t="n">
+      <c r="CG1" s="1">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1" t="n">
+      <c r="CH1" s="1">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1" t="n">
+      <c r="CI1" s="1">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1" t="n">
+      <c r="CJ1" s="1">
         <v>46112</v>
       </c>
-      <c r="CK1" s="1" t="n">
+      <c r="CK1" s="1">
         <v>46023</v>
       </c>
-      <c r="CL1" s="1" t="n">
+      <c r="CL1" s="1">
         <v>46024</v>
       </c>
-      <c r="CM1" s="1" t="n">
+      <c r="CM1" s="1">
         <v>46025</v>
       </c>
-      <c r="CN1" s="1" t="n">
+      <c r="CN1" s="1">
         <v>46026</v>
       </c>
-      <c r="CO1" s="1" t="n">
+      <c r="CO1" s="1">
         <v>46027</v>
       </c>
-      <c r="CP1" s="1" t="n">
+      <c r="CP1" s="1">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="1" t="n">
+      <c r="CQ1" s="1">
         <v>46113</v>
       </c>
-      <c r="CR1" s="1" t="n">
+      <c r="CR1" s="1">
         <v>46114</v>
       </c>
-      <c r="CS1" s="1" t="n">
+      <c r="CS1" s="1">
         <v>46115</v>
       </c>
-      <c r="CT1" s="1" t="n">
+      <c r="CT1" s="1">
         <v>46116</v>
       </c>
-      <c r="CU1" s="1" t="n">
+      <c r="CU1" s="1">
         <v>46117</v>
       </c>
-      <c r="CV1" s="1" t="n">
+      <c r="CV1" s="1">
         <v>46118</v>
       </c>
-      <c r="CW1" s="1" t="n">
+      <c r="CW1" s="1">
         <v>46119</v>
       </c>
-      <c r="CX1" s="1" t="n">
+      <c r="CX1" s="1">
         <v>46120</v>
       </c>
-      <c r="CY1" s="1" t="n">
+      <c r="CY1" s="1">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="1" t="n">
+      <c r="CZ1" s="1">
         <v>46122</v>
       </c>
-      <c r="DA1" s="1" t="n">
+      <c r="DA1" s="1">
         <v>46123</v>
       </c>
-      <c r="DB1" s="1" t="n">
+      <c r="DB1" s="1">
         <v>46124</v>
       </c>
-      <c r="DC1" s="1" t="n">
+      <c r="DC1" s="1">
         <v>46125</v>
       </c>
-      <c r="DD1" s="1" t="n">
+      <c r="DD1" s="1">
         <v>46126</v>
       </c>
-      <c r="DE1" s="1" t="n">
+      <c r="DE1" s="1">
         <v>46127</v>
       </c>
-      <c r="DF1" s="1" t="n">
+      <c r="DF1" s="1">
         <v>46128</v>
       </c>
-      <c r="DG1" s="1" t="n">
+      <c r="DG1" s="1">
         <v>46129</v>
       </c>
-      <c r="DH1" s="1" t="n">
+      <c r="DH1" s="1">
         <v>46130</v>
       </c>
-      <c r="DI1" s="1" t="n">
+      <c r="DI1" s="1">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="1" t="n">
+      <c r="DJ1" s="1">
         <v>46132</v>
       </c>
-      <c r="DK1" s="1" t="n">
+      <c r="DK1" s="1">
         <v>46133</v>
       </c>
-      <c r="DL1" s="1" t="n">
+      <c r="DL1" s="1">
         <v>46134</v>
       </c>
-      <c r="DM1" s="1" t="n">
+      <c r="DM1" s="1">
         <v>46135</v>
       </c>
-      <c r="DN1" s="1" t="n">
+      <c r="DN1" s="1">
         <v>46136</v>
       </c>
-      <c r="DO1" s="1" t="n">
+      <c r="DO1" s="1">
         <v>46137</v>
       </c>
-      <c r="DP1" s="1" t="n">
+      <c r="DP1" s="1">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="1" t="n">
+      <c r="DQ1" s="1">
         <v>46139</v>
       </c>
-      <c r="DR1" s="1" t="n">
+      <c r="DR1" s="1">
         <v>46140</v>
       </c>
-      <c r="DS1" s="1" t="n">
+      <c r="DS1" s="1">
         <v>46141</v>
       </c>
-      <c r="DT1" s="1" t="n">
+      <c r="DT1" s="1">
         <v>46142</v>
       </c>
-      <c r="DU1" s="1" t="n">
+      <c r="DU1" s="1">
         <v>46143</v>
       </c>
-      <c r="DV1" s="1" t="n">
+      <c r="DV1" s="1">
         <v>46144</v>
       </c>
-      <c r="DW1" s="1" t="n">
+      <c r="DW1" s="1">
         <v>46145</v>
       </c>
-      <c r="DX1" s="1" t="n">
+      <c r="DX1" s="1">
         <v>46146</v>
       </c>
-      <c r="DY1" s="1" t="n">
+      <c r="DY1" s="1">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="1" t="n">
+      <c r="DZ1" s="1">
         <v>46148</v>
       </c>
-      <c r="EA1" s="1" t="n">
+      <c r="EA1" s="1">
         <v>46149</v>
       </c>
-      <c r="EB1" s="1" t="n">
+      <c r="EB1" s="1">
         <v>46150</v>
       </c>
-      <c r="EC1" s="1" t="n">
+      <c r="EC1" s="1">
         <v>46151</v>
       </c>
-      <c r="ED1" s="1" t="n">
+      <c r="ED1" s="1">
         <v>46152</v>
       </c>
-      <c r="EE1" s="1" t="n">
+      <c r="EE1" s="1">
         <v>46153</v>
       </c>
-      <c r="EF1" s="1" t="n">
+      <c r="EF1" s="1">
         <v>46154</v>
       </c>
-      <c r="EG1" s="1" t="n">
+      <c r="EG1" s="1">
         <v>46155</v>
       </c>
-      <c r="EH1" s="1" t="n">
+      <c r="EH1" s="1">
         <v>46156</v>
       </c>
-      <c r="EI1" s="1" t="n">
+      <c r="EI1" s="1">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="1" t="n">
+      <c r="EJ1" s="1">
         <v>46158</v>
       </c>
-      <c r="EK1" s="1" t="n">
+      <c r="EK1" s="1">
         <v>46159</v>
       </c>
-      <c r="EL1" s="1" t="n">
+      <c r="EL1" s="1">
         <v>46160</v>
       </c>
-      <c r="EM1" s="1" t="n">
+      <c r="EM1" s="1">
         <v>46161</v>
       </c>
-      <c r="EN1" s="1" t="n">
+      <c r="EN1" s="1">
         <v>46162</v>
       </c>
-      <c r="EO1" s="1" t="n">
+      <c r="EO1" s="1">
         <v>46163</v>
       </c>
-      <c r="EP1" s="1" t="n">
+      <c r="EP1" s="1">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="1" t="n">
+      <c r="EQ1" s="1">
         <v>46165</v>
       </c>
-      <c r="ER1" s="1" t="n">
+      <c r="ER1" s="1">
         <v>46166</v>
       </c>
-      <c r="ES1" s="1" t="n">
+      <c r="ES1" s="1">
         <v>46167</v>
       </c>
-      <c r="ET1" s="1" t="n">
+      <c r="ET1" s="1">
         <v>46168</v>
       </c>
-      <c r="EU1" s="1" t="n">
+      <c r="EU1" s="1">
         <v>46169</v>
       </c>
-      <c r="EV1" s="1" t="n">
+      <c r="EV1" s="1">
         <v>46170</v>
       </c>
-      <c r="EW1" s="1" t="n">
+      <c r="EW1" s="1">
         <v>46171</v>
       </c>
-      <c r="EX1" s="1" t="n">
+      <c r="EX1" s="1">
         <v>46172</v>
       </c>
-      <c r="EY1" s="1" t="n">
+      <c r="EY1" s="1">
         <v>46173</v>
       </c>
-      <c r="EZ1" s="1" t="n">
+      <c r="EZ1" s="1">
         <v>46022</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Data Analyst</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Jose Gomez</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>L639</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>ON NS</t>
-        </is>
-      </c>
-      <c r="CK2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CL2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CM2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="CN2" s="3" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="CO2" s="3" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="CP2" s="3" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="EZ2" s="2" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cuenta de tony agregada
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -1,66 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1+D CRUD\inboundoutbound\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B2275E-1CEF-447C-A419-71F82033294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operations_best_opt" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations_best_opt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>TEAM</t>
-  </si>
-  <si>
-    <t>ROLE</t>
-  </si>
-  <si>
-    <t>NAME</t>
-  </si>
-  <si>
-    <t>BADGE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -75,23 +59,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -379,481 +424,632 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EZ1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:EZ3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:156" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>BADGE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n">
         <v>46029</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1" s="1" t="n">
         <v>46030</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1" s="1" t="n">
         <v>46031</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1" s="1" t="n">
         <v>46032</v>
       </c>
-      <c r="I1" s="1">
+      <c r="I1" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="J1" s="1">
+      <c r="J1" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="K1" s="1">
+      <c r="K1" s="1" t="n">
         <v>46035</v>
       </c>
-      <c r="L1" s="1">
+      <c r="L1" s="1" t="n">
         <v>46036</v>
       </c>
-      <c r="M1" s="1">
+      <c r="M1" s="1" t="n">
         <v>46037</v>
       </c>
-      <c r="N1" s="1">
+      <c r="N1" s="1" t="n">
         <v>46038</v>
       </c>
-      <c r="O1" s="1">
+      <c r="O1" s="1" t="n">
         <v>46039</v>
       </c>
-      <c r="P1" s="1">
+      <c r="P1" s="1" t="n">
         <v>46040</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="Q1" s="1" t="n">
         <v>46041</v>
       </c>
-      <c r="R1" s="1">
+      <c r="R1" s="1" t="n">
         <v>46042</v>
       </c>
-      <c r="S1" s="1">
+      <c r="S1" s="1" t="n">
         <v>46043</v>
       </c>
-      <c r="T1" s="1">
+      <c r="T1" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="U1" s="1">
+      <c r="U1" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="V1" s="1">
+      <c r="V1" s="1" t="n">
         <v>46046</v>
       </c>
-      <c r="W1" s="1">
+      <c r="W1" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="X1" s="1">
+      <c r="X1" s="1" t="n">
         <v>46048</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="Y1" s="1" t="n">
         <v>46049</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Z1" s="1" t="n">
         <v>46050</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AA1" s="1" t="n">
         <v>46051</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AB1" s="1" t="n">
         <v>46052</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AC1" s="1" t="n">
         <v>46053</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AD1" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AE1" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AF1" s="1" t="n">
         <v>46056</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AG1" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AH1" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="AI1" s="1" t="n">
         <v>46059</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AJ1" s="1" t="n">
         <v>46060</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AK1" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AL1" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AM1" s="1" t="n">
         <v>46063</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AN1" s="1" t="n">
         <v>46064</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AO1" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AP1" s="1" t="n">
         <v>46066</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AQ1" s="1" t="n">
         <v>46067</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AR1" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AS1" s="1" t="n">
         <v>46069</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AT1" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AU1" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AV1" s="1" t="n">
         <v>46072</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AW1" s="1" t="n">
         <v>46073</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AX1" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AY1" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AZ1" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="BA1" s="1" t="n">
         <v>46077</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="BB1" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="BC1" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="BD1" s="1" t="n">
         <v>46080</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="BE1" s="1" t="n">
         <v>46081</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="BF1" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="BG1" s="1" t="n">
         <v>46083</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="BH1" s="1" t="n">
         <v>46084</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="BI1" s="1" t="n">
         <v>46085</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BJ1" s="1" t="n">
         <v>46086</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BK1" s="1" t="n">
         <v>46087</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BL1" s="1" t="n">
         <v>46088</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BM1" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="BN1" s="1">
+      <c r="BN1" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="BO1" s="1">
+      <c r="BO1" s="1" t="n">
         <v>46091</v>
       </c>
-      <c r="BP1" s="1">
+      <c r="BP1" s="1" t="n">
         <v>46092</v>
       </c>
-      <c r="BQ1" s="1">
+      <c r="BQ1" s="1" t="n">
         <v>46093</v>
       </c>
-      <c r="BR1" s="1">
+      <c r="BR1" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="BS1" s="1">
+      <c r="BS1" s="1" t="n">
         <v>46095</v>
       </c>
-      <c r="BT1" s="1">
+      <c r="BT1" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="BU1" s="1">
+      <c r="BU1" s="1" t="n">
         <v>46097</v>
       </c>
-      <c r="BV1" s="1">
+      <c r="BV1" s="1" t="n">
         <v>46098</v>
       </c>
-      <c r="BW1" s="1">
+      <c r="BW1" s="1" t="n">
         <v>46099</v>
       </c>
-      <c r="BX1" s="1">
+      <c r="BX1" s="1" t="n">
         <v>46100</v>
       </c>
-      <c r="BY1" s="1">
+      <c r="BY1" s="1" t="n">
         <v>46101</v>
       </c>
-      <c r="BZ1" s="1">
+      <c r="BZ1" s="1" t="n">
         <v>46102</v>
       </c>
-      <c r="CA1" s="1">
+      <c r="CA1" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="CB1" s="1">
+      <c r="CB1" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="CC1" s="1">
+      <c r="CC1" s="1" t="n">
         <v>46105</v>
       </c>
-      <c r="CD1" s="1">
+      <c r="CD1" s="1" t="n">
         <v>46106</v>
       </c>
-      <c r="CE1" s="1">
+      <c r="CE1" s="1" t="n">
         <v>46107</v>
       </c>
-      <c r="CF1" s="1">
+      <c r="CF1" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="CG1" s="1">
+      <c r="CG1" s="1" t="n">
         <v>46109</v>
       </c>
-      <c r="CH1" s="1">
+      <c r="CH1" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="CI1" s="1">
+      <c r="CI1" s="1" t="n">
         <v>46111</v>
       </c>
-      <c r="CJ1" s="1">
+      <c r="CJ1" s="1" t="n">
         <v>46112</v>
       </c>
-      <c r="CK1" s="1">
+      <c r="CK1" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="CL1" s="1">
+      <c r="CL1" s="1" t="n">
         <v>46024</v>
       </c>
-      <c r="CM1" s="1">
+      <c r="CM1" s="1" t="n">
         <v>46025</v>
       </c>
-      <c r="CN1" s="1">
+      <c r="CN1" s="1" t="n">
         <v>46026</v>
       </c>
-      <c r="CO1" s="1">
+      <c r="CO1" s="1" t="n">
         <v>46027</v>
       </c>
-      <c r="CP1" s="1">
+      <c r="CP1" s="1" t="n">
         <v>46028</v>
       </c>
-      <c r="CQ1" s="1">
+      <c r="CQ1" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="CR1" s="1">
+      <c r="CR1" s="1" t="n">
         <v>46114</v>
       </c>
-      <c r="CS1" s="1">
+      <c r="CS1" s="1" t="n">
         <v>46115</v>
       </c>
-      <c r="CT1" s="1">
+      <c r="CT1" s="1" t="n">
         <v>46116</v>
       </c>
-      <c r="CU1" s="1">
+      <c r="CU1" s="1" t="n">
         <v>46117</v>
       </c>
-      <c r="CV1" s="1">
+      <c r="CV1" s="1" t="n">
         <v>46118</v>
       </c>
-      <c r="CW1" s="1">
+      <c r="CW1" s="1" t="n">
         <v>46119</v>
       </c>
-      <c r="CX1" s="1">
+      <c r="CX1" s="1" t="n">
         <v>46120</v>
       </c>
-      <c r="CY1" s="1">
+      <c r="CY1" s="1" t="n">
         <v>46121</v>
       </c>
-      <c r="CZ1" s="1">
+      <c r="CZ1" s="1" t="n">
         <v>46122</v>
       </c>
-      <c r="DA1" s="1">
+      <c r="DA1" s="1" t="n">
         <v>46123</v>
       </c>
-      <c r="DB1" s="1">
+      <c r="DB1" s="1" t="n">
         <v>46124</v>
       </c>
-      <c r="DC1" s="1">
+      <c r="DC1" s="1" t="n">
         <v>46125</v>
       </c>
-      <c r="DD1" s="1">
+      <c r="DD1" s="1" t="n">
         <v>46126</v>
       </c>
-      <c r="DE1" s="1">
+      <c r="DE1" s="1" t="n">
         <v>46127</v>
       </c>
-      <c r="DF1" s="1">
+      <c r="DF1" s="1" t="n">
         <v>46128</v>
       </c>
-      <c r="DG1" s="1">
+      <c r="DG1" s="1" t="n">
         <v>46129</v>
       </c>
-      <c r="DH1" s="1">
+      <c r="DH1" s="1" t="n">
         <v>46130</v>
       </c>
-      <c r="DI1" s="1">
+      <c r="DI1" s="1" t="n">
         <v>46131</v>
       </c>
-      <c r="DJ1" s="1">
+      <c r="DJ1" s="1" t="n">
         <v>46132</v>
       </c>
-      <c r="DK1" s="1">
+      <c r="DK1" s="1" t="n">
         <v>46133</v>
       </c>
-      <c r="DL1" s="1">
+      <c r="DL1" s="1" t="n">
         <v>46134</v>
       </c>
-      <c r="DM1" s="1">
+      <c r="DM1" s="1" t="n">
         <v>46135</v>
       </c>
-      <c r="DN1" s="1">
+      <c r="DN1" s="1" t="n">
         <v>46136</v>
       </c>
-      <c r="DO1" s="1">
+      <c r="DO1" s="1" t="n">
         <v>46137</v>
       </c>
-      <c r="DP1" s="1">
+      <c r="DP1" s="1" t="n">
         <v>46138</v>
       </c>
-      <c r="DQ1" s="1">
+      <c r="DQ1" s="1" t="n">
         <v>46139</v>
       </c>
-      <c r="DR1" s="1">
+      <c r="DR1" s="1" t="n">
         <v>46140</v>
       </c>
-      <c r="DS1" s="1">
+      <c r="DS1" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="DT1" s="1">
+      <c r="DT1" s="1" t="n">
         <v>46142</v>
       </c>
-      <c r="DU1" s="1">
+      <c r="DU1" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="DV1" s="1">
+      <c r="DV1" s="1" t="n">
         <v>46144</v>
       </c>
-      <c r="DW1" s="1">
+      <c r="DW1" s="1" t="n">
         <v>46145</v>
       </c>
-      <c r="DX1" s="1">
+      <c r="DX1" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="DY1" s="1">
+      <c r="DY1" s="1" t="n">
         <v>46147</v>
       </c>
-      <c r="DZ1" s="1">
+      <c r="DZ1" s="1" t="n">
         <v>46148</v>
       </c>
-      <c r="EA1" s="1">
+      <c r="EA1" s="1" t="n">
         <v>46149</v>
       </c>
-      <c r="EB1" s="1">
+      <c r="EB1" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="EC1" s="1">
+      <c r="EC1" s="1" t="n">
         <v>46151</v>
       </c>
-      <c r="ED1" s="1">
+      <c r="ED1" s="1" t="n">
         <v>46152</v>
       </c>
-      <c r="EE1" s="1">
+      <c r="EE1" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="EF1" s="1">
+      <c r="EF1" s="1" t="n">
         <v>46154</v>
       </c>
-      <c r="EG1" s="1">
+      <c r="EG1" s="1" t="n">
         <v>46155</v>
       </c>
-      <c r="EH1" s="1">
+      <c r="EH1" s="1" t="n">
         <v>46156</v>
       </c>
-      <c r="EI1" s="1">
+      <c r="EI1" s="1" t="n">
         <v>46157</v>
       </c>
-      <c r="EJ1" s="1">
+      <c r="EJ1" s="1" t="n">
         <v>46158</v>
       </c>
-      <c r="EK1" s="1">
+      <c r="EK1" s="1" t="n">
         <v>46159</v>
       </c>
-      <c r="EL1" s="1">
+      <c r="EL1" s="1" t="n">
         <v>46160</v>
       </c>
-      <c r="EM1" s="1">
+      <c r="EM1" s="1" t="n">
         <v>46161</v>
       </c>
-      <c r="EN1" s="1">
+      <c r="EN1" s="1" t="n">
         <v>46162</v>
       </c>
-      <c r="EO1" s="1">
+      <c r="EO1" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="EP1" s="1">
+      <c r="EP1" s="1" t="n">
         <v>46164</v>
       </c>
-      <c r="EQ1" s="1">
+      <c r="EQ1" s="1" t="n">
         <v>46165</v>
       </c>
-      <c r="ER1" s="1">
+      <c r="ER1" s="1" t="n">
         <v>46166</v>
       </c>
-      <c r="ES1" s="1">
+      <c r="ES1" s="1" t="n">
         <v>46167</v>
       </c>
-      <c r="ET1" s="1">
+      <c r="ET1" s="1" t="n">
         <v>46168</v>
       </c>
-      <c r="EU1" s="1">
+      <c r="EU1" s="1" t="n">
         <v>46169</v>
       </c>
-      <c r="EV1" s="1">
+      <c r="EV1" s="1" t="n">
         <v>46170</v>
       </c>
-      <c r="EW1" s="1">
+      <c r="EW1" s="1" t="n">
         <v>46171</v>
       </c>
-      <c r="EX1" s="1">
+      <c r="EX1" s="1" t="n">
         <v>46172</v>
       </c>
-      <c r="EY1" s="1">
+      <c r="EY1" s="1" t="n">
         <v>46173</v>
       </c>
-      <c r="EZ1" s="1">
+      <c r="EZ1" s="1" t="n">
         <v>46022</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mauricio Arrieta</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>L123</t>
+        </is>
+      </c>
+      <c r="CC2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CD2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CE2" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CF2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CG2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CH2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CI2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CJ2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CK2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CL2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CM2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CN2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CQ2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CR2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="CS2" s="3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Joram Herrera</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TP0904</t>
+        </is>
+      </c>
+      <c r="CB3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CC3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CD3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CE3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CF3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="CG3" s="2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Primera frase de buenas practicas aplicadas, toca hacer pruebas exahustivas
</commit_message>
<xml_diff>
--- a/PlanStaffNewmont.xlsx
+++ b/PlanStaffNewmont.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -59,11 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EZ3"/>
+  <dimension ref="A1:HI3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="5" max="13"/>
@@ -912,6 +914,189 @@
       <c r="EZ1" s="1" t="n">
         <v>46022</v>
       </c>
+      <c r="FA1" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="FB1" s="4" t="n">
+        <v>46175</v>
+      </c>
+      <c r="FC1" s="4" t="n">
+        <v>46176</v>
+      </c>
+      <c r="FD1" s="4" t="n">
+        <v>46177</v>
+      </c>
+      <c r="FE1" s="4" t="n">
+        <v>46178</v>
+      </c>
+      <c r="FF1" s="4" t="n">
+        <v>46179</v>
+      </c>
+      <c r="FG1" s="4" t="n">
+        <v>46180</v>
+      </c>
+      <c r="FH1" s="4" t="n">
+        <v>46181</v>
+      </c>
+      <c r="FI1" s="4" t="n">
+        <v>46182</v>
+      </c>
+      <c r="FJ1" s="4" t="n">
+        <v>46183</v>
+      </c>
+      <c r="FK1" s="4" t="n">
+        <v>46184</v>
+      </c>
+      <c r="FL1" s="4" t="n">
+        <v>46185</v>
+      </c>
+      <c r="FM1" s="4" t="n">
+        <v>46186</v>
+      </c>
+      <c r="FN1" s="4" t="n">
+        <v>46187</v>
+      </c>
+      <c r="FO1" s="4" t="n">
+        <v>46188</v>
+      </c>
+      <c r="FP1" s="4" t="n">
+        <v>46189</v>
+      </c>
+      <c r="FQ1" s="4" t="n">
+        <v>46190</v>
+      </c>
+      <c r="FR1" s="4" t="n">
+        <v>46191</v>
+      </c>
+      <c r="FS1" s="4" t="n">
+        <v>46192</v>
+      </c>
+      <c r="FT1" s="4" t="n">
+        <v>46193</v>
+      </c>
+      <c r="FU1" s="4" t="n">
+        <v>46194</v>
+      </c>
+      <c r="FV1" s="4" t="n">
+        <v>46195</v>
+      </c>
+      <c r="FW1" s="4" t="n">
+        <v>46196</v>
+      </c>
+      <c r="FX1" s="4" t="n">
+        <v>46197</v>
+      </c>
+      <c r="FY1" s="4" t="n">
+        <v>46198</v>
+      </c>
+      <c r="FZ1" s="4" t="n">
+        <v>46199</v>
+      </c>
+      <c r="GA1" s="4" t="n">
+        <v>46200</v>
+      </c>
+      <c r="GB1" s="4" t="n">
+        <v>46201</v>
+      </c>
+      <c r="GC1" s="4" t="n">
+        <v>46202</v>
+      </c>
+      <c r="GD1" s="4" t="n">
+        <v>46203</v>
+      </c>
+      <c r="GE1" s="4" t="n">
+        <v>46204</v>
+      </c>
+      <c r="GF1" s="4" t="n">
+        <v>46205</v>
+      </c>
+      <c r="GG1" s="4" t="n">
+        <v>46206</v>
+      </c>
+      <c r="GH1" s="4" t="n">
+        <v>46207</v>
+      </c>
+      <c r="GI1" s="4" t="n">
+        <v>46208</v>
+      </c>
+      <c r="GJ1" s="4" t="n">
+        <v>46209</v>
+      </c>
+      <c r="GK1" s="4" t="n">
+        <v>46210</v>
+      </c>
+      <c r="GL1" s="4" t="n">
+        <v>46211</v>
+      </c>
+      <c r="GM1" s="4" t="n">
+        <v>46212</v>
+      </c>
+      <c r="GN1" s="4" t="n">
+        <v>46213</v>
+      </c>
+      <c r="GO1" s="4" t="n">
+        <v>46214</v>
+      </c>
+      <c r="GP1" s="4" t="n">
+        <v>46215</v>
+      </c>
+      <c r="GQ1" s="4" t="n">
+        <v>46216</v>
+      </c>
+      <c r="GR1" s="4" t="n">
+        <v>46217</v>
+      </c>
+      <c r="GS1" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="GT1" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="GU1" s="4" t="n">
+        <v>46220</v>
+      </c>
+      <c r="GV1" s="4" t="n">
+        <v>46221</v>
+      </c>
+      <c r="GW1" s="4" t="n">
+        <v>46222</v>
+      </c>
+      <c r="GX1" s="4" t="n">
+        <v>46223</v>
+      </c>
+      <c r="GY1" s="4" t="n">
+        <v>46224</v>
+      </c>
+      <c r="GZ1" s="4" t="n">
+        <v>46225</v>
+      </c>
+      <c r="HA1" s="4" t="n">
+        <v>46226</v>
+      </c>
+      <c r="HB1" s="4" t="n">
+        <v>46227</v>
+      </c>
+      <c r="HC1" s="4" t="n">
+        <v>46228</v>
+      </c>
+      <c r="HD1" s="4" t="n">
+        <v>46229</v>
+      </c>
+      <c r="HE1" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="HF1" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="HG1" s="4" t="n">
+        <v>46232</v>
+      </c>
+      <c r="HH1" s="4" t="n">
+        <v>46233</v>
+      </c>
+      <c r="HI1" s="4" t="n">
+        <v>46234</v>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">

</xml_diff>